<commit_message>
Worked on Take Over.
</commit_message>
<xml_diff>
--- a/Take Over/Anlage_10_Vorlage_Kostenplan_GBW25.xlsx
+++ b/Take Over/Anlage_10_Vorlage_Kostenplan_GBW25.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\ScrewDriversMFG\Take Over\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7794B4B1-5F94-4C57-92DC-BC254C8357CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BEE8792-E016-4405-AFB0-E6AE8A0334A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38880" yWindow="1470" windowWidth="36525" windowHeight="27375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="77340" yWindow="1755" windowWidth="37560" windowHeight="27375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kosten_Planung" sheetId="1" r:id="rId1"/>
@@ -1547,28 +1547,56 @@
     <xf numFmtId="17" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="4" fontId="2" fillId="11" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1576,15 +1604,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1606,12 +1625,6 @@
     <xf numFmtId="44" fontId="16" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1630,35 +1643,34 @@
     <xf numFmtId="44" fontId="5" fillId="4" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="2" fillId="11" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="4" fontId="2" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1680,18 +1692,6 @@
     <xf numFmtId="44" fontId="16" fillId="7" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Prozent" xfId="2" builtinId="5"/>
@@ -1988,38 +1988,38 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="197"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="151"/>
-      <c r="H2" s="151"/>
-      <c r="I2" s="151"/>
-      <c r="J2" s="151"/>
-      <c r="K2" s="151"/>
-      <c r="L2" s="151"/>
-      <c r="M2" s="151"/>
-      <c r="N2" s="151"/>
-      <c r="O2" s="151"/>
-      <c r="P2" s="151"/>
-      <c r="Q2" s="151"/>
-      <c r="R2" s="151"/>
-      <c r="S2" s="151"/>
-      <c r="T2" s="151"/>
-      <c r="U2" s="151"/>
-      <c r="V2" s="151"/>
-      <c r="W2" s="151"/>
-      <c r="X2" s="151"/>
-      <c r="Y2" s="151"/>
-      <c r="Z2" s="151"/>
-      <c r="AA2" s="151"/>
-      <c r="AB2" s="151"/>
-      <c r="AC2" s="151"/>
+      <c r="F2" s="147"/>
+      <c r="G2" s="147"/>
+      <c r="H2" s="147"/>
+      <c r="I2" s="147"/>
+      <c r="J2" s="147"/>
+      <c r="K2" s="147"/>
+      <c r="L2" s="147"/>
+      <c r="M2" s="147"/>
+      <c r="N2" s="147"/>
+      <c r="O2" s="147"/>
+      <c r="P2" s="147"/>
+      <c r="Q2" s="147"/>
+      <c r="R2" s="147"/>
+      <c r="S2" s="147"/>
+      <c r="T2" s="147"/>
+      <c r="U2" s="147"/>
+      <c r="V2" s="147"/>
+      <c r="W2" s="147"/>
+      <c r="X2" s="147"/>
+      <c r="Y2" s="147"/>
+      <c r="Z2" s="147"/>
+      <c r="AA2" s="147"/>
+      <c r="AB2" s="147"/>
+      <c r="AC2" s="147"/>
     </row>
     <row r="3" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="184"/>
-      <c r="C3" s="186" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="186"/>
+      <c r="B3" s="149"/>
+      <c r="C3" s="151" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="151"/>
       <c r="E3" s="72">
         <v>1</v>
       </c>
@@ -2097,9 +2097,9 @@
     </row>
     <row r="4" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="185"/>
-      <c r="C4" s="187"/>
-      <c r="D4" s="187"/>
+      <c r="B4" s="150"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="152"/>
       <c r="E4" s="38" t="s">
         <v>1</v>
       </c>
@@ -2172,10 +2172,10 @@
       <c r="AB4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="AC4" s="187" t="s">
+      <c r="AC4" s="152" t="s">
         <v>2</v>
       </c>
-      <c r="AD4" s="162" t="s">
+      <c r="AD4" s="157" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2186,32 +2186,32 @@
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="E5" s="182"/>
-      <c r="F5" s="151"/>
-      <c r="G5" s="151"/>
-      <c r="H5" s="151"/>
-      <c r="I5" s="151"/>
-      <c r="J5" s="151"/>
-      <c r="K5" s="151"/>
-      <c r="L5" s="151"/>
-      <c r="M5" s="151"/>
-      <c r="N5" s="151"/>
-      <c r="O5" s="151"/>
-      <c r="P5" s="151"/>
-      <c r="Q5" s="151"/>
-      <c r="R5" s="151"/>
-      <c r="S5" s="151"/>
-      <c r="T5" s="151"/>
-      <c r="U5" s="151"/>
-      <c r="V5" s="151"/>
-      <c r="W5" s="151"/>
-      <c r="X5" s="151"/>
-      <c r="Y5" s="151"/>
-      <c r="Z5" s="151"/>
-      <c r="AA5" s="151"/>
-      <c r="AB5" s="151"/>
-      <c r="AC5" s="187"/>
-      <c r="AD5" s="162"/>
+      <c r="E5" s="158"/>
+      <c r="F5" s="147"/>
+      <c r="G5" s="147"/>
+      <c r="H5" s="147"/>
+      <c r="I5" s="147"/>
+      <c r="J5" s="147"/>
+      <c r="K5" s="147"/>
+      <c r="L5" s="147"/>
+      <c r="M5" s="147"/>
+      <c r="N5" s="147"/>
+      <c r="O5" s="147"/>
+      <c r="P5" s="147"/>
+      <c r="Q5" s="147"/>
+      <c r="R5" s="147"/>
+      <c r="S5" s="147"/>
+      <c r="T5" s="147"/>
+      <c r="U5" s="147"/>
+      <c r="V5" s="147"/>
+      <c r="W5" s="147"/>
+      <c r="X5" s="147"/>
+      <c r="Y5" s="147"/>
+      <c r="Z5" s="147"/>
+      <c r="AA5" s="147"/>
+      <c r="AB5" s="147"/>
+      <c r="AC5" s="152"/>
+      <c r="AD5" s="157"/>
     </row>
     <row r="6" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -2224,32 +2224,32 @@
       <c r="D6" s="68" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="157" t="s">
+      <c r="E6" s="159" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="157"/>
-      <c r="G6" s="157"/>
-      <c r="H6" s="157"/>
-      <c r="I6" s="157"/>
-      <c r="J6" s="157"/>
-      <c r="K6" s="157"/>
-      <c r="L6" s="157"/>
-      <c r="M6" s="157"/>
-      <c r="N6" s="157"/>
-      <c r="O6" s="157"/>
-      <c r="P6" s="157"/>
-      <c r="Q6" s="157"/>
-      <c r="R6" s="157"/>
-      <c r="S6" s="157"/>
-      <c r="T6" s="157"/>
-      <c r="U6" s="157"/>
-      <c r="V6" s="157"/>
-      <c r="W6" s="157"/>
-      <c r="X6" s="157"/>
-      <c r="Y6" s="157"/>
-      <c r="Z6" s="157"/>
-      <c r="AA6" s="157"/>
-      <c r="AB6" s="157"/>
+      <c r="F6" s="159"/>
+      <c r="G6" s="159"/>
+      <c r="H6" s="159"/>
+      <c r="I6" s="159"/>
+      <c r="J6" s="159"/>
+      <c r="K6" s="159"/>
+      <c r="L6" s="159"/>
+      <c r="M6" s="159"/>
+      <c r="N6" s="159"/>
+      <c r="O6" s="159"/>
+      <c r="P6" s="159"/>
+      <c r="Q6" s="159"/>
+      <c r="R6" s="159"/>
+      <c r="S6" s="159"/>
+      <c r="T6" s="159"/>
+      <c r="U6" s="159"/>
+      <c r="V6" s="159"/>
+      <c r="W6" s="159"/>
+      <c r="X6" s="159"/>
+      <c r="Y6" s="159"/>
+      <c r="Z6" s="159"/>
+      <c r="AA6" s="159"/>
+      <c r="AB6" s="159"/>
       <c r="AC6" s="61"/>
       <c r="AD6" s="89"/>
     </row>
@@ -2341,7 +2341,7 @@
         <f>SUM(E7:AB7)*D7</f>
         <v>0</v>
       </c>
-      <c r="AD7" s="171">
+      <c r="AD7" s="161">
         <v>0</v>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
         <f t="shared" ref="AC8:AC24" si="1">SUM(E8:AB8)</f>
         <v>0</v>
       </c>
-      <c r="AD8" s="172"/>
+      <c r="AD8" s="162"/>
     </row>
     <row r="9" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2547,7 +2547,7 @@
         <f>SUM(E9:AB9)*D9</f>
         <v>0</v>
       </c>
-      <c r="AD9" s="171">
+      <c r="AD9" s="161">
         <v>0</v>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD10" s="172"/>
+      <c r="AD10" s="162"/>
     </row>
     <row r="11" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
@@ -2753,7 +2753,7 @@
         <f>SUM(E11:AB11)*D11</f>
         <v>0</v>
       </c>
-      <c r="AD11" s="171">
+      <c r="AD11" s="161">
         <v>0</v>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD12" s="172"/>
+      <c r="AD12" s="162"/>
     </row>
     <row r="13" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
@@ -2959,7 +2959,7 @@
         <f>SUM(E13:AB13)*D13</f>
         <v>0</v>
       </c>
-      <c r="AD13" s="171">
+      <c r="AD13" s="161">
         <v>0</v>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD14" s="172"/>
+      <c r="AD14" s="162"/>
     </row>
     <row r="15" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
@@ -3165,7 +3165,7 @@
         <f>SUM(E15:AB15)*D15</f>
         <v>0</v>
       </c>
-      <c r="AD15" s="171">
+      <c r="AD15" s="161">
         <v>0</v>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD16" s="172"/>
+      <c r="AD16" s="162"/>
     </row>
     <row r="17" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -3371,7 +3371,7 @@
         <f>SUM(E17:AB17)*D17</f>
         <v>0</v>
       </c>
-      <c r="AD17" s="171">
+      <c r="AD17" s="161">
         <v>0</v>
       </c>
     </row>
@@ -3487,7 +3487,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD18" s="172"/>
+      <c r="AD18" s="162"/>
     </row>
     <row r="19" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
@@ -3577,7 +3577,7 @@
         <f>SUM(E19:AB19)*D19</f>
         <v>0</v>
       </c>
-      <c r="AD19" s="171">
+      <c r="AD19" s="161">
         <v>0</v>
       </c>
     </row>
@@ -3693,7 +3693,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD20" s="172"/>
+      <c r="AD20" s="162"/>
     </row>
     <row r="21" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
@@ -3783,7 +3783,7 @@
         <f>SUM(E21:AB21)*D21</f>
         <v>0</v>
       </c>
-      <c r="AD21" s="171">
+      <c r="AD21" s="161">
         <v>0</v>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD22" s="172"/>
+      <c r="AD22" s="162"/>
     </row>
     <row r="23" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
@@ -4008,7 +4008,7 @@
         <f t="shared" ref="AC23" si="10">SUM(E23:AB23)</f>
         <v>0</v>
       </c>
-      <c r="AD23" s="179" t="s">
+      <c r="AD23" s="163" t="s">
         <v>45</v>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD24" s="180"/>
+      <c r="AD24" s="164"/>
     </row>
     <row r="25" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
@@ -4276,32 +4276,32 @@
       <c r="D27" s="68" t="s">
         <v>37</v>
       </c>
-      <c r="E27" s="157" t="s">
+      <c r="E27" s="159" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="154"/>
-      <c r="G27" s="154"/>
-      <c r="H27" s="154"/>
-      <c r="I27" s="154"/>
-      <c r="J27" s="154"/>
-      <c r="K27" s="154"/>
-      <c r="L27" s="154"/>
-      <c r="M27" s="154"/>
-      <c r="N27" s="154"/>
-      <c r="O27" s="154"/>
-      <c r="P27" s="154"/>
-      <c r="Q27" s="154"/>
-      <c r="R27" s="154"/>
-      <c r="S27" s="154"/>
-      <c r="T27" s="154"/>
-      <c r="U27" s="154"/>
-      <c r="V27" s="154"/>
-      <c r="W27" s="154"/>
-      <c r="X27" s="154"/>
-      <c r="Y27" s="154"/>
-      <c r="Z27" s="154"/>
-      <c r="AA27" s="154"/>
-      <c r="AB27" s="154"/>
+      <c r="F27" s="160"/>
+      <c r="G27" s="160"/>
+      <c r="H27" s="160"/>
+      <c r="I27" s="160"/>
+      <c r="J27" s="160"/>
+      <c r="K27" s="160"/>
+      <c r="L27" s="160"/>
+      <c r="M27" s="160"/>
+      <c r="N27" s="160"/>
+      <c r="O27" s="160"/>
+      <c r="P27" s="160"/>
+      <c r="Q27" s="160"/>
+      <c r="R27" s="160"/>
+      <c r="S27" s="160"/>
+      <c r="T27" s="160"/>
+      <c r="U27" s="160"/>
+      <c r="V27" s="160"/>
+      <c r="W27" s="160"/>
+      <c r="X27" s="160"/>
+      <c r="Y27" s="160"/>
+      <c r="Z27" s="160"/>
+      <c r="AA27" s="160"/>
+      <c r="AB27" s="160"/>
       <c r="AC27" s="61"/>
       <c r="AD27" s="89"/>
     </row>
@@ -4393,7 +4393,7 @@
         <f>SUM(E28:AB28)*D28</f>
         <v>0</v>
       </c>
-      <c r="AD28" s="171">
+      <c r="AD28" s="161">
         <v>0</v>
       </c>
     </row>
@@ -4509,7 +4509,7 @@
         <f t="shared" ref="AC29" si="14">SUM(E29:AB29)</f>
         <v>0</v>
       </c>
-      <c r="AD29" s="172"/>
+      <c r="AD29" s="162"/>
     </row>
     <row r="30" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
@@ -4599,7 +4599,7 @@
         <f>SUM(E30:AB30)*D30</f>
         <v>0</v>
       </c>
-      <c r="AD30" s="171">
+      <c r="AD30" s="161">
         <v>0</v>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
         <f t="shared" ref="AC31" si="16">SUM(E31:AB31)</f>
         <v>0</v>
       </c>
-      <c r="AD31" s="172"/>
+      <c r="AD31" s="162"/>
     </row>
     <row r="32" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
@@ -4805,7 +4805,7 @@
         <f>SUM(E32:AB32)*D32</f>
         <v>0</v>
       </c>
-      <c r="AD32" s="171">
+      <c r="AD32" s="161">
         <v>0</v>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
         <f t="shared" ref="AC33" si="18">SUM(E33:AB33)</f>
         <v>0</v>
       </c>
-      <c r="AD33" s="172"/>
+      <c r="AD33" s="162"/>
     </row>
     <row r="34" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
@@ -5011,7 +5011,7 @@
         <f>SUM(E34:AB34)*D34</f>
         <v>0</v>
       </c>
-      <c r="AD34" s="181">
+      <c r="AD34" s="165">
         <v>0</v>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
         <f t="shared" ref="AC35" si="20">SUM(E35:AB35)</f>
         <v>0</v>
       </c>
-      <c r="AD35" s="172"/>
+      <c r="AD35" s="162"/>
     </row>
     <row r="36" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
@@ -5217,7 +5217,7 @@
         <f>SUM(E36:AB36)*D36</f>
         <v>0</v>
       </c>
-      <c r="AD36" s="171">
+      <c r="AD36" s="161">
         <v>0</v>
       </c>
     </row>
@@ -5333,7 +5333,7 @@
         <f t="shared" ref="AC37" si="22">SUM(E37:AB37)</f>
         <v>0</v>
       </c>
-      <c r="AD37" s="172"/>
+      <c r="AD37" s="162"/>
     </row>
     <row r="38" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -5423,7 +5423,7 @@
         <f>SUM(E38:AB38)*D38</f>
         <v>0</v>
       </c>
-      <c r="AD38" s="171">
+      <c r="AD38" s="161">
         <v>0</v>
       </c>
     </row>
@@ -5539,7 +5539,7 @@
         <f t="shared" ref="AC39" si="24">SUM(E39:AB39)</f>
         <v>0</v>
       </c>
-      <c r="AD39" s="172"/>
+      <c r="AD39" s="162"/>
     </row>
     <row r="40" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
@@ -5629,7 +5629,7 @@
         <f>SUM(E40:AB40)*D40</f>
         <v>0</v>
       </c>
-      <c r="AD40" s="171">
+      <c r="AD40" s="161">
         <v>0</v>
       </c>
     </row>
@@ -5745,7 +5745,7 @@
         <f t="shared" ref="AC41:AC43" si="26">SUM(E41:AB41)</f>
         <v>0</v>
       </c>
-      <c r="AD41" s="172"/>
+      <c r="AD41" s="162"/>
     </row>
     <row r="42" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
@@ -5854,7 +5854,7 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-      <c r="AD42" s="162" t="s">
+      <c r="AD42" s="157" t="s">
         <v>45</v>
       </c>
     </row>
@@ -5965,7 +5965,7 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-      <c r="AD43" s="162"/>
+      <c r="AD43" s="157"/>
     </row>
     <row r="44" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
@@ -6118,42 +6118,42 @@
       </c>
       <c r="C46" s="66"/>
       <c r="D46" s="66"/>
-      <c r="E46" s="157" t="s">
+      <c r="E46" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="F46" s="154"/>
-      <c r="G46" s="154"/>
-      <c r="H46" s="154"/>
-      <c r="I46" s="154"/>
-      <c r="J46" s="154"/>
-      <c r="K46" s="154"/>
-      <c r="L46" s="154"/>
-      <c r="M46" s="154"/>
-      <c r="N46" s="154"/>
-      <c r="O46" s="154"/>
-      <c r="P46" s="154"/>
-      <c r="Q46" s="154"/>
-      <c r="R46" s="154"/>
-      <c r="S46" s="154"/>
-      <c r="T46" s="154"/>
-      <c r="U46" s="154"/>
-      <c r="V46" s="154"/>
-      <c r="W46" s="154"/>
-      <c r="X46" s="154"/>
-      <c r="Y46" s="154"/>
-      <c r="Z46" s="154"/>
-      <c r="AA46" s="154"/>
-      <c r="AB46" s="154"/>
+      <c r="F46" s="160"/>
+      <c r="G46" s="160"/>
+      <c r="H46" s="160"/>
+      <c r="I46" s="160"/>
+      <c r="J46" s="160"/>
+      <c r="K46" s="160"/>
+      <c r="L46" s="160"/>
+      <c r="M46" s="160"/>
+      <c r="N46" s="160"/>
+      <c r="O46" s="160"/>
+      <c r="P46" s="160"/>
+      <c r="Q46" s="160"/>
+      <c r="R46" s="160"/>
+      <c r="S46" s="160"/>
+      <c r="T46" s="160"/>
+      <c r="U46" s="160"/>
+      <c r="V46" s="160"/>
+      <c r="W46" s="160"/>
+      <c r="X46" s="160"/>
+      <c r="Y46" s="160"/>
+      <c r="Z46" s="160"/>
+      <c r="AA46" s="160"/>
+      <c r="AB46" s="160"/>
       <c r="AC46" s="61"/>
       <c r="AD46" s="89"/>
     </row>
     <row r="47" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
-      <c r="B47" s="158" t="s">
+      <c r="B47" s="166" t="s">
         <v>40</v>
       </c>
-      <c r="C47" s="159"/>
-      <c r="D47" s="159"/>
+      <c r="C47" s="167"/>
+      <c r="D47" s="167"/>
       <c r="E47" s="12">
         <v>0</v>
       </c>
@@ -6236,11 +6236,11 @@
     </row>
     <row r="48" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
-      <c r="B48" s="160" t="s">
+      <c r="B48" s="153" t="s">
         <v>46</v>
       </c>
-      <c r="C48" s="161"/>
-      <c r="D48" s="161"/>
+      <c r="C48" s="154"/>
+      <c r="D48" s="154"/>
       <c r="E48" s="15">
         <v>0</v>
       </c>
@@ -6323,11 +6323,11 @@
     </row>
     <row r="49" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
-      <c r="B49" s="160" t="s">
+      <c r="B49" s="153" t="s">
         <v>47</v>
       </c>
-      <c r="C49" s="161"/>
-      <c r="D49" s="161"/>
+      <c r="C49" s="154"/>
+      <c r="D49" s="154"/>
       <c r="E49" s="15">
         <v>0</v>
       </c>
@@ -6410,11 +6410,11 @@
     </row>
     <row r="50" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
-      <c r="B50" s="160" t="s">
+      <c r="B50" s="153" t="s">
         <v>43</v>
       </c>
-      <c r="C50" s="161"/>
-      <c r="D50" s="161"/>
+      <c r="C50" s="154"/>
+      <c r="D50" s="154"/>
       <c r="E50" s="18">
         <v>0</v>
       </c>
@@ -6641,47 +6641,47 @@
     </row>
     <row r="53" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
-      <c r="B53" s="155" t="s">
+      <c r="B53" s="188" t="s">
         <v>15</v>
       </c>
-      <c r="C53" s="156"/>
-      <c r="D53" s="156"/>
-      <c r="E53" s="157" t="s">
+      <c r="C53" s="189"/>
+      <c r="D53" s="189"/>
+      <c r="E53" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="F53" s="154"/>
-      <c r="G53" s="154"/>
-      <c r="H53" s="154"/>
-      <c r="I53" s="154"/>
-      <c r="J53" s="154"/>
-      <c r="K53" s="154"/>
-      <c r="L53" s="154"/>
-      <c r="M53" s="154"/>
-      <c r="N53" s="154"/>
-      <c r="O53" s="154"/>
-      <c r="P53" s="154"/>
-      <c r="Q53" s="154"/>
-      <c r="R53" s="154"/>
-      <c r="S53" s="154"/>
-      <c r="T53" s="154"/>
-      <c r="U53" s="154"/>
-      <c r="V53" s="154"/>
-      <c r="W53" s="154"/>
-      <c r="X53" s="154"/>
-      <c r="Y53" s="154"/>
-      <c r="Z53" s="154"/>
-      <c r="AA53" s="154"/>
-      <c r="AB53" s="154"/>
+      <c r="F53" s="160"/>
+      <c r="G53" s="160"/>
+      <c r="H53" s="160"/>
+      <c r="I53" s="160"/>
+      <c r="J53" s="160"/>
+      <c r="K53" s="160"/>
+      <c r="L53" s="160"/>
+      <c r="M53" s="160"/>
+      <c r="N53" s="160"/>
+      <c r="O53" s="160"/>
+      <c r="P53" s="160"/>
+      <c r="Q53" s="160"/>
+      <c r="R53" s="160"/>
+      <c r="S53" s="160"/>
+      <c r="T53" s="160"/>
+      <c r="U53" s="160"/>
+      <c r="V53" s="160"/>
+      <c r="W53" s="160"/>
+      <c r="X53" s="160"/>
+      <c r="Y53" s="160"/>
+      <c r="Z53" s="160"/>
+      <c r="AA53" s="160"/>
+      <c r="AB53" s="160"/>
       <c r="AC53" s="61"/>
       <c r="AD53" s="89"/>
     </row>
     <row r="54" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="158" t="s">
+      <c r="B54" s="166" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="159"/>
-      <c r="D54" s="159"/>
+      <c r="C54" s="167"/>
+      <c r="D54" s="167"/>
       <c r="E54" s="12">
         <v>0</v>
       </c>
@@ -6764,11 +6764,11 @@
     </row>
     <row r="55" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
-      <c r="B55" s="160" t="s">
+      <c r="B55" s="153" t="s">
         <v>17</v>
       </c>
-      <c r="C55" s="161"/>
-      <c r="D55" s="161"/>
+      <c r="C55" s="154"/>
+      <c r="D55" s="154"/>
       <c r="E55" s="15">
         <v>0</v>
       </c>
@@ -6851,11 +6851,11 @@
     </row>
     <row r="56" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
-      <c r="B56" s="160" t="s">
+      <c r="B56" s="153" t="s">
         <v>18</v>
       </c>
-      <c r="C56" s="161"/>
-      <c r="D56" s="161"/>
+      <c r="C56" s="154"/>
+      <c r="D56" s="154"/>
       <c r="E56" s="15">
         <v>0</v>
       </c>
@@ -6938,11 +6938,11 @@
     </row>
     <row r="57" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
-      <c r="B57" s="160" t="s">
+      <c r="B57" s="153" t="s">
         <v>18</v>
       </c>
-      <c r="C57" s="161"/>
-      <c r="D57" s="161"/>
+      <c r="C57" s="154"/>
+      <c r="D57" s="154"/>
       <c r="E57" s="18">
         <v>0</v>
       </c>
@@ -7169,47 +7169,47 @@
     </row>
     <row r="60" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
-      <c r="B60" s="166" t="s">
+      <c r="B60" s="171" t="s">
         <v>19</v>
       </c>
-      <c r="C60" s="167"/>
-      <c r="D60" s="167"/>
-      <c r="E60" s="157" t="s">
+      <c r="C60" s="172"/>
+      <c r="D60" s="172"/>
+      <c r="E60" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="F60" s="154"/>
-      <c r="G60" s="154"/>
-      <c r="H60" s="154"/>
-      <c r="I60" s="154"/>
-      <c r="J60" s="154"/>
-      <c r="K60" s="154"/>
-      <c r="L60" s="154"/>
-      <c r="M60" s="154"/>
-      <c r="N60" s="154"/>
-      <c r="O60" s="154"/>
-      <c r="P60" s="154"/>
-      <c r="Q60" s="154"/>
-      <c r="R60" s="154"/>
-      <c r="S60" s="154"/>
-      <c r="T60" s="154"/>
-      <c r="U60" s="154"/>
-      <c r="V60" s="154"/>
-      <c r="W60" s="154"/>
-      <c r="X60" s="154"/>
-      <c r="Y60" s="154"/>
-      <c r="Z60" s="154"/>
-      <c r="AA60" s="154"/>
-      <c r="AB60" s="154"/>
+      <c r="F60" s="160"/>
+      <c r="G60" s="160"/>
+      <c r="H60" s="160"/>
+      <c r="I60" s="160"/>
+      <c r="J60" s="160"/>
+      <c r="K60" s="160"/>
+      <c r="L60" s="160"/>
+      <c r="M60" s="160"/>
+      <c r="N60" s="160"/>
+      <c r="O60" s="160"/>
+      <c r="P60" s="160"/>
+      <c r="Q60" s="160"/>
+      <c r="R60" s="160"/>
+      <c r="S60" s="160"/>
+      <c r="T60" s="160"/>
+      <c r="U60" s="160"/>
+      <c r="V60" s="160"/>
+      <c r="W60" s="160"/>
+      <c r="X60" s="160"/>
+      <c r="Y60" s="160"/>
+      <c r="Z60" s="160"/>
+      <c r="AA60" s="160"/>
+      <c r="AB60" s="160"/>
       <c r="AC60" s="61"/>
       <c r="AD60" s="89"/>
     </row>
     <row r="61" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
-      <c r="B61" s="158" t="s">
+      <c r="B61" s="166" t="s">
         <v>20</v>
       </c>
-      <c r="C61" s="159"/>
-      <c r="D61" s="159"/>
+      <c r="C61" s="167"/>
+      <c r="D61" s="167"/>
       <c r="E61" s="12">
         <v>0</v>
       </c>
@@ -7292,11 +7292,11 @@
     </row>
     <row r="62" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
-      <c r="B62" s="160" t="s">
+      <c r="B62" s="153" t="s">
         <v>62</v>
       </c>
-      <c r="C62" s="161"/>
-      <c r="D62" s="161"/>
+      <c r="C62" s="154"/>
+      <c r="D62" s="154"/>
       <c r="E62" s="15">
         <v>0</v>
       </c>
@@ -7379,11 +7379,11 @@
     </row>
     <row r="63" spans="1:30" ht="15" x14ac:dyDescent="0.3">
       <c r="A63" s="3"/>
-      <c r="B63" s="160" t="s">
+      <c r="B63" s="153" t="s">
         <v>21</v>
       </c>
-      <c r="C63" s="161"/>
-      <c r="D63" s="161"/>
+      <c r="C63" s="154"/>
+      <c r="D63" s="154"/>
       <c r="E63" s="15">
         <v>0</v>
       </c>
@@ -7715,7 +7715,7 @@
         <f t="shared" ref="AC66:AC67" si="37">SUM(E66:AB66)</f>
         <v>0</v>
       </c>
-      <c r="AD66" s="169"/>
+      <c r="AD66" s="174"/>
     </row>
     <row r="67" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
@@ -7824,7 +7824,7 @@
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="AD67" s="162"/>
+      <c r="AD67" s="157"/>
     </row>
     <row r="68" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
@@ -7933,7 +7933,7 @@
         <f t="shared" si="34"/>
         <v>0</v>
       </c>
-      <c r="AD68" s="162"/>
+      <c r="AD68" s="157"/>
     </row>
     <row r="69" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
@@ -8039,7 +8039,7 @@
         <v>0</v>
       </c>
       <c r="AC69" s="112"/>
-      <c r="AD69" s="163"/>
+      <c r="AD69" s="168"/>
     </row>
     <row r="70" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
@@ -8080,31 +8080,31 @@
       </c>
       <c r="C71" s="60"/>
       <c r="D71" s="60"/>
-      <c r="E71" s="153"/>
-      <c r="F71" s="154"/>
-      <c r="G71" s="154"/>
-      <c r="H71" s="154"/>
-      <c r="I71" s="154"/>
-      <c r="J71" s="154"/>
-      <c r="K71" s="154"/>
-      <c r="L71" s="154"/>
-      <c r="M71" s="154"/>
-      <c r="N71" s="154"/>
-      <c r="O71" s="154"/>
-      <c r="P71" s="154"/>
-      <c r="Q71" s="154"/>
-      <c r="R71" s="154"/>
-      <c r="S71" s="154"/>
-      <c r="T71" s="154"/>
-      <c r="U71" s="154"/>
-      <c r="V71" s="154"/>
-      <c r="W71" s="154"/>
-      <c r="X71" s="154"/>
-      <c r="Y71" s="154"/>
-      <c r="Z71" s="154"/>
-      <c r="AA71" s="154"/>
-      <c r="AB71" s="154"/>
-      <c r="AC71" s="154"/>
+      <c r="E71" s="187"/>
+      <c r="F71" s="160"/>
+      <c r="G71" s="160"/>
+      <c r="H71" s="160"/>
+      <c r="I71" s="160"/>
+      <c r="J71" s="160"/>
+      <c r="K71" s="160"/>
+      <c r="L71" s="160"/>
+      <c r="M71" s="160"/>
+      <c r="N71" s="160"/>
+      <c r="O71" s="160"/>
+      <c r="P71" s="160"/>
+      <c r="Q71" s="160"/>
+      <c r="R71" s="160"/>
+      <c r="S71" s="160"/>
+      <c r="T71" s="160"/>
+      <c r="U71" s="160"/>
+      <c r="V71" s="160"/>
+      <c r="W71" s="160"/>
+      <c r="X71" s="160"/>
+      <c r="Y71" s="160"/>
+      <c r="Z71" s="160"/>
+      <c r="AA71" s="160"/>
+      <c r="AB71" s="160"/>
+      <c r="AC71" s="160"/>
       <c r="AD71" s="89"/>
     </row>
     <row r="72" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
@@ -8116,35 +8116,35 @@
       <c r="D72" s="142">
         <v>0</v>
       </c>
-      <c r="E72" s="175">
+      <c r="E72" s="178">
         <f>D72-E73</f>
         <v>0</v>
       </c>
-      <c r="F72" s="176"/>
-      <c r="G72" s="176"/>
-      <c r="H72" s="176"/>
-      <c r="I72" s="176"/>
-      <c r="J72" s="176"/>
-      <c r="K72" s="176"/>
-      <c r="L72" s="176"/>
-      <c r="M72" s="176"/>
-      <c r="N72" s="176"/>
-      <c r="O72" s="176"/>
-      <c r="P72" s="176"/>
-      <c r="Q72" s="176"/>
-      <c r="R72" s="176"/>
-      <c r="S72" s="176"/>
-      <c r="T72" s="176"/>
-      <c r="U72" s="176"/>
-      <c r="V72" s="176"/>
-      <c r="W72" s="176"/>
-      <c r="X72" s="176"/>
-      <c r="Y72" s="176"/>
-      <c r="Z72" s="176"/>
-      <c r="AA72" s="176"/>
-      <c r="AB72" s="176"/>
-      <c r="AC72" s="176"/>
-      <c r="AD72" s="171">
+      <c r="F72" s="179"/>
+      <c r="G72" s="179"/>
+      <c r="H72" s="179"/>
+      <c r="I72" s="179"/>
+      <c r="J72" s="179"/>
+      <c r="K72" s="179"/>
+      <c r="L72" s="179"/>
+      <c r="M72" s="179"/>
+      <c r="N72" s="179"/>
+      <c r="O72" s="179"/>
+      <c r="P72" s="179"/>
+      <c r="Q72" s="179"/>
+      <c r="R72" s="179"/>
+      <c r="S72" s="179"/>
+      <c r="T72" s="179"/>
+      <c r="U72" s="179"/>
+      <c r="V72" s="179"/>
+      <c r="W72" s="179"/>
+      <c r="X72" s="179"/>
+      <c r="Y72" s="179"/>
+      <c r="Z72" s="179"/>
+      <c r="AA72" s="179"/>
+      <c r="AB72" s="179"/>
+      <c r="AC72" s="179"/>
+      <c r="AD72" s="161">
         <v>0</v>
       </c>
     </row>
@@ -8157,35 +8157,35 @@
       <c r="D73" s="143">
         <v>0</v>
       </c>
-      <c r="E73" s="177">
+      <c r="E73" s="180">
         <f>D72*D73</f>
         <v>0</v>
       </c>
-      <c r="F73" s="178"/>
-      <c r="G73" s="178"/>
-      <c r="H73" s="178"/>
-      <c r="I73" s="178"/>
-      <c r="J73" s="178"/>
-      <c r="K73" s="178"/>
-      <c r="L73" s="178"/>
-      <c r="M73" s="178"/>
-      <c r="N73" s="178"/>
-      <c r="O73" s="178"/>
-      <c r="P73" s="178"/>
-      <c r="Q73" s="178"/>
-      <c r="R73" s="178"/>
-      <c r="S73" s="178"/>
-      <c r="T73" s="178"/>
-      <c r="U73" s="178"/>
-      <c r="V73" s="178"/>
-      <c r="W73" s="178"/>
-      <c r="X73" s="178"/>
-      <c r="Y73" s="178"/>
-      <c r="Z73" s="178"/>
-      <c r="AA73" s="178"/>
-      <c r="AB73" s="178"/>
-      <c r="AC73" s="178"/>
-      <c r="AD73" s="172"/>
+      <c r="F73" s="181"/>
+      <c r="G73" s="181"/>
+      <c r="H73" s="181"/>
+      <c r="I73" s="181"/>
+      <c r="J73" s="181"/>
+      <c r="K73" s="181"/>
+      <c r="L73" s="181"/>
+      <c r="M73" s="181"/>
+      <c r="N73" s="181"/>
+      <c r="O73" s="181"/>
+      <c r="P73" s="181"/>
+      <c r="Q73" s="181"/>
+      <c r="R73" s="181"/>
+      <c r="S73" s="181"/>
+      <c r="T73" s="181"/>
+      <c r="U73" s="181"/>
+      <c r="V73" s="181"/>
+      <c r="W73" s="181"/>
+      <c r="X73" s="181"/>
+      <c r="Y73" s="181"/>
+      <c r="Z73" s="181"/>
+      <c r="AA73" s="181"/>
+      <c r="AB73" s="181"/>
+      <c r="AC73" s="181"/>
+      <c r="AD73" s="162"/>
     </row>
     <row r="74" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
@@ -8198,76 +8198,76 @@
       <c r="D74" s="126">
         <v>0</v>
       </c>
-      <c r="E74" s="196">
+      <c r="E74" s="204">
         <f>D74-E75</f>
         <v>0</v>
       </c>
-      <c r="F74" s="196"/>
-      <c r="G74" s="196"/>
-      <c r="H74" s="196"/>
-      <c r="I74" s="196"/>
-      <c r="J74" s="196"/>
-      <c r="K74" s="196"/>
-      <c r="L74" s="196"/>
-      <c r="M74" s="196"/>
-      <c r="N74" s="196"/>
-      <c r="O74" s="196"/>
-      <c r="P74" s="196"/>
-      <c r="Q74" s="196"/>
-      <c r="R74" s="196"/>
-      <c r="S74" s="196"/>
-      <c r="T74" s="196"/>
-      <c r="U74" s="196"/>
-      <c r="V74" s="196"/>
-      <c r="W74" s="196"/>
-      <c r="X74" s="196"/>
-      <c r="Y74" s="196"/>
-      <c r="Z74" s="196"/>
-      <c r="AA74" s="196"/>
-      <c r="AB74" s="196"/>
-      <c r="AC74" s="196"/>
-      <c r="AD74" s="192">
+      <c r="F74" s="204"/>
+      <c r="G74" s="204"/>
+      <c r="H74" s="204"/>
+      <c r="I74" s="204"/>
+      <c r="J74" s="204"/>
+      <c r="K74" s="204"/>
+      <c r="L74" s="204"/>
+      <c r="M74" s="204"/>
+      <c r="N74" s="204"/>
+      <c r="O74" s="204"/>
+      <c r="P74" s="204"/>
+      <c r="Q74" s="204"/>
+      <c r="R74" s="204"/>
+      <c r="S74" s="204"/>
+      <c r="T74" s="204"/>
+      <c r="U74" s="204"/>
+      <c r="V74" s="204"/>
+      <c r="W74" s="204"/>
+      <c r="X74" s="204"/>
+      <c r="Y74" s="204"/>
+      <c r="Z74" s="204"/>
+      <c r="AA74" s="204"/>
+      <c r="AB74" s="204"/>
+      <c r="AC74" s="204"/>
+      <c r="AD74" s="200">
         <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
-      <c r="B75" s="201" t="s">
+      <c r="B75" s="195" t="s">
         <v>57</v>
       </c>
-      <c r="C75" s="202"/>
+      <c r="C75" s="196"/>
       <c r="D75" s="127">
         <v>0</v>
       </c>
-      <c r="E75" s="194">
+      <c r="E75" s="202">
         <f>D74*D75</f>
         <v>0</v>
       </c>
-      <c r="F75" s="194"/>
-      <c r="G75" s="194"/>
-      <c r="H75" s="194"/>
-      <c r="I75" s="194"/>
-      <c r="J75" s="194"/>
-      <c r="K75" s="194"/>
-      <c r="L75" s="194"/>
-      <c r="M75" s="194"/>
-      <c r="N75" s="194"/>
-      <c r="O75" s="194"/>
-      <c r="P75" s="194"/>
-      <c r="Q75" s="194"/>
-      <c r="R75" s="194"/>
-      <c r="S75" s="194"/>
-      <c r="T75" s="194"/>
-      <c r="U75" s="194"/>
-      <c r="V75" s="194"/>
-      <c r="W75" s="194"/>
-      <c r="X75" s="194"/>
-      <c r="Y75" s="194"/>
-      <c r="Z75" s="194"/>
-      <c r="AA75" s="194"/>
-      <c r="AB75" s="194"/>
-      <c r="AC75" s="194"/>
-      <c r="AD75" s="193"/>
+      <c r="F75" s="202"/>
+      <c r="G75" s="202"/>
+      <c r="H75" s="202"/>
+      <c r="I75" s="202"/>
+      <c r="J75" s="202"/>
+      <c r="K75" s="202"/>
+      <c r="L75" s="202"/>
+      <c r="M75" s="202"/>
+      <c r="N75" s="202"/>
+      <c r="O75" s="202"/>
+      <c r="P75" s="202"/>
+      <c r="Q75" s="202"/>
+      <c r="R75" s="202"/>
+      <c r="S75" s="202"/>
+      <c r="T75" s="202"/>
+      <c r="U75" s="202"/>
+      <c r="V75" s="202"/>
+      <c r="W75" s="202"/>
+      <c r="X75" s="202"/>
+      <c r="Y75" s="202"/>
+      <c r="Z75" s="202"/>
+      <c r="AA75" s="202"/>
+      <c r="AB75" s="202"/>
+      <c r="AC75" s="202"/>
+      <c r="AD75" s="201"/>
     </row>
     <row r="76" spans="1:30" ht="15" x14ac:dyDescent="0.3">
       <c r="A76" s="3"/>
@@ -8280,35 +8280,35 @@
       <c r="D76" s="117">
         <v>0</v>
       </c>
-      <c r="E76" s="195">
+      <c r="E76" s="203">
         <f>D76</f>
         <v>0</v>
       </c>
-      <c r="F76" s="195"/>
-      <c r="G76" s="195"/>
-      <c r="H76" s="195"/>
-      <c r="I76" s="195"/>
-      <c r="J76" s="195"/>
-      <c r="K76" s="195"/>
-      <c r="L76" s="195"/>
-      <c r="M76" s="195"/>
-      <c r="N76" s="195"/>
-      <c r="O76" s="195"/>
-      <c r="P76" s="195"/>
-      <c r="Q76" s="195"/>
-      <c r="R76" s="195"/>
-      <c r="S76" s="195"/>
-      <c r="T76" s="195"/>
-      <c r="U76" s="195"/>
-      <c r="V76" s="195"/>
-      <c r="W76" s="195"/>
-      <c r="X76" s="195"/>
-      <c r="Y76" s="195"/>
-      <c r="Z76" s="195"/>
-      <c r="AA76" s="195"/>
-      <c r="AB76" s="195"/>
-      <c r="AC76" s="195"/>
-      <c r="AD76" s="162" t="s">
+      <c r="F76" s="203"/>
+      <c r="G76" s="203"/>
+      <c r="H76" s="203"/>
+      <c r="I76" s="203"/>
+      <c r="J76" s="203"/>
+      <c r="K76" s="203"/>
+      <c r="L76" s="203"/>
+      <c r="M76" s="203"/>
+      <c r="N76" s="203"/>
+      <c r="O76" s="203"/>
+      <c r="P76" s="203"/>
+      <c r="Q76" s="203"/>
+      <c r="R76" s="203"/>
+      <c r="S76" s="203"/>
+      <c r="T76" s="203"/>
+      <c r="U76" s="203"/>
+      <c r="V76" s="203"/>
+      <c r="W76" s="203"/>
+      <c r="X76" s="203"/>
+      <c r="Y76" s="203"/>
+      <c r="Z76" s="203"/>
+      <c r="AA76" s="203"/>
+      <c r="AB76" s="203"/>
+      <c r="AC76" s="203"/>
+      <c r="AD76" s="157" t="s">
         <v>54</v>
       </c>
     </row>
@@ -8319,67 +8319,67 @@
       </c>
       <c r="C77" s="129"/>
       <c r="D77" s="129"/>
-      <c r="E77" s="203"/>
-      <c r="F77" s="204"/>
-      <c r="G77" s="204"/>
-      <c r="H77" s="204"/>
-      <c r="I77" s="204"/>
-      <c r="J77" s="204"/>
-      <c r="K77" s="204"/>
-      <c r="L77" s="204"/>
-      <c r="M77" s="204"/>
-      <c r="N77" s="204"/>
-      <c r="O77" s="204"/>
-      <c r="P77" s="204"/>
-      <c r="Q77" s="204"/>
-      <c r="R77" s="204"/>
-      <c r="S77" s="204"/>
-      <c r="T77" s="204"/>
-      <c r="U77" s="204"/>
-      <c r="V77" s="204"/>
-      <c r="W77" s="204"/>
-      <c r="X77" s="204"/>
-      <c r="Y77" s="204"/>
-      <c r="Z77" s="204"/>
-      <c r="AA77" s="204"/>
-      <c r="AB77" s="204"/>
+      <c r="E77" s="190"/>
+      <c r="F77" s="191"/>
+      <c r="G77" s="191"/>
+      <c r="H77" s="191"/>
+      <c r="I77" s="191"/>
+      <c r="J77" s="191"/>
+      <c r="K77" s="191"/>
+      <c r="L77" s="191"/>
+      <c r="M77" s="191"/>
+      <c r="N77" s="191"/>
+      <c r="O77" s="191"/>
+      <c r="P77" s="191"/>
+      <c r="Q77" s="191"/>
+      <c r="R77" s="191"/>
+      <c r="S77" s="191"/>
+      <c r="T77" s="191"/>
+      <c r="U77" s="191"/>
+      <c r="V77" s="191"/>
+      <c r="W77" s="191"/>
+      <c r="X77" s="191"/>
+      <c r="Y77" s="191"/>
+      <c r="Z77" s="191"/>
+      <c r="AA77" s="191"/>
+      <c r="AB77" s="191"/>
       <c r="AC77" s="130">
         <f>D74+D76+D72</f>
         <v>0</v>
       </c>
-      <c r="AD77" s="162"/>
+      <c r="AD77" s="157"/>
     </row>
     <row r="78" spans="1:30" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="5"/>
-      <c r="B78" s="198" t="s">
+      <c r="B78" s="192" t="s">
         <v>26</v>
       </c>
-      <c r="C78" s="199"/>
+      <c r="C78" s="193"/>
       <c r="D78" s="131"/>
-      <c r="E78" s="200"/>
-      <c r="F78" s="199"/>
-      <c r="G78" s="199"/>
-      <c r="H78" s="199"/>
-      <c r="I78" s="199"/>
-      <c r="J78" s="199"/>
-      <c r="K78" s="199"/>
-      <c r="L78" s="199"/>
-      <c r="M78" s="199"/>
-      <c r="N78" s="199"/>
-      <c r="O78" s="199"/>
-      <c r="P78" s="199"/>
-      <c r="Q78" s="199"/>
-      <c r="R78" s="199"/>
-      <c r="S78" s="199"/>
-      <c r="T78" s="199"/>
-      <c r="U78" s="199"/>
-      <c r="V78" s="199"/>
-      <c r="W78" s="199"/>
-      <c r="X78" s="199"/>
-      <c r="Y78" s="199"/>
-      <c r="Z78" s="199"/>
-      <c r="AA78" s="199"/>
-      <c r="AB78" s="199"/>
+      <c r="E78" s="194"/>
+      <c r="F78" s="193"/>
+      <c r="G78" s="193"/>
+      <c r="H78" s="193"/>
+      <c r="I78" s="193"/>
+      <c r="J78" s="193"/>
+      <c r="K78" s="193"/>
+      <c r="L78" s="193"/>
+      <c r="M78" s="193"/>
+      <c r="N78" s="193"/>
+      <c r="O78" s="193"/>
+      <c r="P78" s="193"/>
+      <c r="Q78" s="193"/>
+      <c r="R78" s="193"/>
+      <c r="S78" s="193"/>
+      <c r="T78" s="193"/>
+      <c r="U78" s="193"/>
+      <c r="V78" s="193"/>
+      <c r="W78" s="193"/>
+      <c r="X78" s="193"/>
+      <c r="Y78" s="193"/>
+      <c r="Z78" s="193"/>
+      <c r="AA78" s="193"/>
+      <c r="AB78" s="193"/>
       <c r="AC78" s="132">
         <f>AC77+AC68</f>
         <v>0</v>
@@ -8453,10 +8453,10 @@
     </row>
     <row r="81" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
-      <c r="B81" s="150" t="s">
+      <c r="B81" s="186" t="s">
         <v>27</v>
       </c>
-      <c r="C81" s="151"/>
+      <c r="C81" s="147"/>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
@@ -8619,10 +8619,10 @@
     </row>
     <row r="86" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
-      <c r="B86" s="152" t="s">
+      <c r="B86" s="146" t="s">
         <v>32</v>
       </c>
-      <c r="C86" s="151"/>
+      <c r="C86" s="147"/>
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
@@ -8651,10 +8651,10 @@
     </row>
     <row r="87" spans="1:29" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
-      <c r="B87" s="188" t="s">
+      <c r="B87" s="155" t="s">
         <v>33</v>
       </c>
-      <c r="C87" s="151"/>
+      <c r="C87" s="147"/>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
@@ -8714,10 +8714,10 @@
     </row>
     <row r="89" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
-      <c r="B89" s="189" t="s">
+      <c r="B89" s="156" t="s">
         <v>56</v>
       </c>
-      <c r="C89" s="151"/>
+      <c r="C89" s="147"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
@@ -8746,10 +8746,10 @@
     </row>
     <row r="90" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A90" s="1"/>
-      <c r="B90" s="183" t="s">
+      <c r="B90" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="C90" s="151"/>
+      <c r="C90" s="147"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
@@ -8778,8 +8778,8 @@
     </row>
     <row r="91" spans="1:29" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
-      <c r="B91" s="151"/>
-      <c r="C91" s="151"/>
+      <c r="B91" s="147"/>
+      <c r="C91" s="147"/>
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
       <c r="G91" s="1"/>
@@ -8839,10 +8839,10 @@
     </row>
     <row r="93" spans="1:29" ht="15" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
-      <c r="B93" s="152" t="s">
+      <c r="B93" s="146" t="s">
         <v>59</v>
       </c>
-      <c r="C93" s="151"/>
+      <c r="C93" s="147"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
       <c r="G93" s="1"/>
@@ -8871,10 +8871,10 @@
     </row>
     <row r="94" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
-      <c r="B94" s="183" t="s">
+      <c r="B94" s="148" t="s">
         <v>55</v>
       </c>
-      <c r="C94" s="151"/>
+      <c r="C94" s="147"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
@@ -8903,8 +8903,8 @@
     </row>
     <row r="95" spans="1:29" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1"/>
-      <c r="B95" s="151"/>
-      <c r="C95" s="151"/>
+      <c r="B95" s="147"/>
+      <c r="C95" s="147"/>
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
@@ -8964,10 +8964,10 @@
     </row>
     <row r="97" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A97" s="1"/>
-      <c r="B97" s="152" t="s">
+      <c r="B97" s="146" t="s">
         <v>66</v>
       </c>
-      <c r="C97" s="151"/>
+      <c r="C97" s="147"/>
       <c r="D97" s="4"/>
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
@@ -8997,10 +8997,10 @@
     </row>
     <row r="98" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A98" s="1"/>
-      <c r="B98" s="190" t="s">
+      <c r="B98" s="198" t="s">
         <v>67</v>
       </c>
-      <c r="C98" s="190"/>
+      <c r="C98" s="198"/>
       <c r="D98" s="1"/>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
@@ -9030,8 +9030,8 @@
     </row>
     <row r="99" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A99" s="1"/>
-      <c r="B99" s="190"/>
-      <c r="C99" s="190"/>
+      <c r="B99" s="198"/>
+      <c r="C99" s="198"/>
       <c r="D99" s="1"/>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
@@ -9092,8 +9092,8 @@
     </row>
     <row r="101" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A101" s="1"/>
-      <c r="B101" s="191"/>
-      <c r="C101" s="151"/>
+      <c r="B101" s="199"/>
+      <c r="C101" s="147"/>
       <c r="D101" s="1"/>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
@@ -38139,6 +38139,55 @@
     </row>
   </sheetData>
   <mergeCells count="65">
+    <mergeCell ref="AD72:AD73"/>
+    <mergeCell ref="E73:AC73"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B98:C99"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="E72:AC72"/>
+    <mergeCell ref="AD74:AD75"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="E75:AC75"/>
+    <mergeCell ref="E76:AC76"/>
+    <mergeCell ref="E74:AC74"/>
+    <mergeCell ref="B94:C95"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B90:C91"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="E2:AC2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="E6:AB6"/>
+    <mergeCell ref="C3:D4"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="E5:AB5"/>
+    <mergeCell ref="E53:AB53"/>
+    <mergeCell ref="E27:AB27"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="E60:AB60"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="E78:AB78"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="AD4:AD5"/>
+    <mergeCell ref="AC4:AC5"/>
+    <mergeCell ref="AD7:AD8"/>
+    <mergeCell ref="AD9:AD10"/>
+    <mergeCell ref="AD21:AD22"/>
+    <mergeCell ref="AD19:AD20"/>
+    <mergeCell ref="AD17:AD18"/>
+    <mergeCell ref="AD15:AD16"/>
+    <mergeCell ref="AD13:AD14"/>
+    <mergeCell ref="AD11:AD12"/>
     <mergeCell ref="AD23:AD24"/>
     <mergeCell ref="E46:AB46"/>
     <mergeCell ref="B50:D50"/>
@@ -38155,55 +38204,6 @@
     <mergeCell ref="E71:AC71"/>
     <mergeCell ref="E77:AB77"/>
     <mergeCell ref="AD66:AD69"/>
-    <mergeCell ref="AD4:AD5"/>
-    <mergeCell ref="AC4:AC5"/>
-    <mergeCell ref="AD7:AD8"/>
-    <mergeCell ref="AD9:AD10"/>
-    <mergeCell ref="AD21:AD22"/>
-    <mergeCell ref="AD19:AD20"/>
-    <mergeCell ref="AD17:AD18"/>
-    <mergeCell ref="AD15:AD16"/>
-    <mergeCell ref="AD13:AD14"/>
-    <mergeCell ref="AD11:AD12"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="E60:AB60"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="E78:AB78"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="E2:AC2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="E6:AB6"/>
-    <mergeCell ref="C3:D4"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="E5:AB5"/>
-    <mergeCell ref="E53:AB53"/>
-    <mergeCell ref="E27:AB27"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="AD72:AD73"/>
-    <mergeCell ref="E73:AC73"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B98:C99"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="E72:AC72"/>
-    <mergeCell ref="AD74:AD75"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="E75:AC75"/>
-    <mergeCell ref="E76:AC76"/>
-    <mergeCell ref="E74:AC74"/>
-    <mergeCell ref="B94:C95"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B90:C91"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B87:C87"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.56333333333333335" bottom="0.44958333333333333" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="52" orientation="landscape" r:id="rId1"/>
@@ -38238,44 +38238,44 @@
   <sheetData>
     <row r="1" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
-      <c r="B1" s="146" t="s">
+      <c r="B1" s="182" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
-      <c r="L1" s="146"/>
-      <c r="M1" s="146"/>
-      <c r="N1" s="146"/>
-      <c r="O1" s="146"/>
-      <c r="P1" s="146"/>
-      <c r="Q1" s="146"/>
-      <c r="R1" s="146"/>
-      <c r="S1" s="146"/>
-      <c r="T1" s="146"/>
-      <c r="U1" s="146"/>
-      <c r="V1" s="146"/>
-      <c r="W1" s="146"/>
-      <c r="X1" s="146"/>
-      <c r="Y1" s="146"/>
-      <c r="Z1" s="146"/>
-      <c r="AA1" s="146"/>
-      <c r="AB1" s="146"/>
-      <c r="AC1" s="146"/>
+      <c r="C1" s="182"/>
+      <c r="D1" s="182"/>
+      <c r="E1" s="182"/>
+      <c r="F1" s="182"/>
+      <c r="G1" s="182"/>
+      <c r="H1" s="182"/>
+      <c r="I1" s="182"/>
+      <c r="J1" s="182"/>
+      <c r="K1" s="182"/>
+      <c r="L1" s="182"/>
+      <c r="M1" s="182"/>
+      <c r="N1" s="182"/>
+      <c r="O1" s="182"/>
+      <c r="P1" s="182"/>
+      <c r="Q1" s="182"/>
+      <c r="R1" s="182"/>
+      <c r="S1" s="182"/>
+      <c r="T1" s="182"/>
+      <c r="U1" s="182"/>
+      <c r="V1" s="182"/>
+      <c r="W1" s="182"/>
+      <c r="X1" s="182"/>
+      <c r="Y1" s="182"/>
+      <c r="Z1" s="182"/>
+      <c r="AA1" s="182"/>
+      <c r="AB1" s="182"/>
+      <c r="AC1" s="182"/>
     </row>
     <row r="2" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="184"/>
-      <c r="C2" s="186" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="186"/>
+      <c r="B2" s="149"/>
+      <c r="C2" s="151" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="151"/>
       <c r="E2" s="72">
         <v>1</v>
       </c>
@@ -38353,9 +38353,9 @@
     </row>
     <row r="3" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="185"/>
-      <c r="C3" s="187"/>
-      <c r="D3" s="187"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="152"/>
+      <c r="D3" s="152"/>
       <c r="E3" s="145">
         <v>46235</v>
       </c>
@@ -38428,10 +38428,10 @@
       <c r="AB3" s="145">
         <v>46935</v>
       </c>
-      <c r="AC3" s="187" t="s">
+      <c r="AC3" s="152" t="s">
         <v>2</v>
       </c>
-      <c r="AD3" s="162" t="s">
+      <c r="AD3" s="157" t="s">
         <v>45</v>
       </c>
     </row>
@@ -38442,32 +38442,32 @@
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="182"/>
-      <c r="F4" s="151"/>
-      <c r="G4" s="151"/>
-      <c r="H4" s="151"/>
-      <c r="I4" s="151"/>
-      <c r="J4" s="151"/>
-      <c r="K4" s="151"/>
-      <c r="L4" s="151"/>
-      <c r="M4" s="151"/>
-      <c r="N4" s="151"/>
-      <c r="O4" s="151"/>
-      <c r="P4" s="151"/>
-      <c r="Q4" s="151"/>
-      <c r="R4" s="151"/>
-      <c r="S4" s="151"/>
-      <c r="T4" s="151"/>
-      <c r="U4" s="151"/>
-      <c r="V4" s="151"/>
-      <c r="W4" s="151"/>
-      <c r="X4" s="151"/>
-      <c r="Y4" s="151"/>
-      <c r="Z4" s="151"/>
-      <c r="AA4" s="151"/>
-      <c r="AB4" s="151"/>
-      <c r="AC4" s="187"/>
-      <c r="AD4" s="162"/>
+      <c r="E4" s="158"/>
+      <c r="F4" s="147"/>
+      <c r="G4" s="147"/>
+      <c r="H4" s="147"/>
+      <c r="I4" s="147"/>
+      <c r="J4" s="147"/>
+      <c r="K4" s="147"/>
+      <c r="L4" s="147"/>
+      <c r="M4" s="147"/>
+      <c r="N4" s="147"/>
+      <c r="O4" s="147"/>
+      <c r="P4" s="147"/>
+      <c r="Q4" s="147"/>
+      <c r="R4" s="147"/>
+      <c r="S4" s="147"/>
+      <c r="T4" s="147"/>
+      <c r="U4" s="147"/>
+      <c r="V4" s="147"/>
+      <c r="W4" s="147"/>
+      <c r="X4" s="147"/>
+      <c r="Y4" s="147"/>
+      <c r="Z4" s="147"/>
+      <c r="AA4" s="147"/>
+      <c r="AB4" s="147"/>
+      <c r="AC4" s="152"/>
+      <c r="AD4" s="157"/>
     </row>
     <row r="5" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
@@ -38480,32 +38480,32 @@
       <c r="D5" s="68" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="157" t="s">
+      <c r="E5" s="159" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="157"/>
-      <c r="G5" s="157"/>
-      <c r="H5" s="157"/>
-      <c r="I5" s="157"/>
-      <c r="J5" s="157"/>
-      <c r="K5" s="157"/>
-      <c r="L5" s="157"/>
-      <c r="M5" s="157"/>
-      <c r="N5" s="157"/>
-      <c r="O5" s="157"/>
-      <c r="P5" s="157"/>
-      <c r="Q5" s="157"/>
-      <c r="R5" s="157"/>
-      <c r="S5" s="157"/>
-      <c r="T5" s="157"/>
-      <c r="U5" s="157"/>
-      <c r="V5" s="157"/>
-      <c r="W5" s="157"/>
-      <c r="X5" s="157"/>
-      <c r="Y5" s="157"/>
-      <c r="Z5" s="157"/>
-      <c r="AA5" s="157"/>
-      <c r="AB5" s="157"/>
+      <c r="F5" s="159"/>
+      <c r="G5" s="159"/>
+      <c r="H5" s="159"/>
+      <c r="I5" s="159"/>
+      <c r="J5" s="159"/>
+      <c r="K5" s="159"/>
+      <c r="L5" s="159"/>
+      <c r="M5" s="159"/>
+      <c r="N5" s="159"/>
+      <c r="O5" s="159"/>
+      <c r="P5" s="159"/>
+      <c r="Q5" s="159"/>
+      <c r="R5" s="159"/>
+      <c r="S5" s="159"/>
+      <c r="T5" s="159"/>
+      <c r="U5" s="159"/>
+      <c r="V5" s="159"/>
+      <c r="W5" s="159"/>
+      <c r="X5" s="159"/>
+      <c r="Y5" s="159"/>
+      <c r="Z5" s="159"/>
+      <c r="AA5" s="159"/>
+      <c r="AB5" s="159"/>
       <c r="AC5" s="61"/>
       <c r="AD5" s="89"/>
     </row>
@@ -38597,7 +38597,7 @@
         <f>SUM(E6:AB6)*D6</f>
         <v>41283</v>
       </c>
-      <c r="AD6" s="171">
+      <c r="AD6" s="161">
         <f>AC6</f>
         <v>41283</v>
       </c>
@@ -38714,7 +38714,7 @@
         <f t="shared" ref="AC7:AC23" si="1">SUM(E7:AB7)</f>
         <v>0</v>
       </c>
-      <c r="AD7" s="172"/>
+      <c r="AD7" s="162"/>
     </row>
     <row r="8" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -38804,7 +38804,7 @@
         <f>SUM(E8:AB8)*D8</f>
         <v>0</v>
       </c>
-      <c r="AD8" s="171">
+      <c r="AD8" s="161">
         <f>AC8</f>
         <v>0</v>
       </c>
@@ -38921,7 +38921,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD9" s="172"/>
+      <c r="AD9" s="162"/>
     </row>
     <row r="10" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
@@ -39011,7 +39011,7 @@
         <f>SUM(E10:AB10)*D10</f>
         <v>0</v>
       </c>
-      <c r="AD10" s="171">
+      <c r="AD10" s="161">
         <v>0</v>
       </c>
     </row>
@@ -39127,7 +39127,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD11" s="172"/>
+      <c r="AD11" s="162"/>
     </row>
     <row r="12" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -39217,7 +39217,7 @@
         <f>SUM(E12:AB12)*D12</f>
         <v>0</v>
       </c>
-      <c r="AD12" s="171">
+      <c r="AD12" s="161">
         <f>AC12</f>
         <v>0</v>
       </c>
@@ -39334,7 +39334,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD13" s="172"/>
+      <c r="AD13" s="162"/>
     </row>
     <row r="14" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -39424,7 +39424,7 @@
         <f>SUM(E14:AB14)*D14</f>
         <v>8580</v>
       </c>
-      <c r="AD14" s="171">
+      <c r="AD14" s="161">
         <f>AC14</f>
         <v>8580</v>
       </c>
@@ -39541,7 +39541,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD15" s="172"/>
+      <c r="AD15" s="162"/>
     </row>
     <row r="16" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
@@ -39631,7 +39631,7 @@
         <f>SUM(E16:AB16)*D16</f>
         <v>4910.4000000000005</v>
       </c>
-      <c r="AD16" s="171">
+      <c r="AD16" s="161">
         <f>AC16</f>
         <v>4910.4000000000005</v>
       </c>
@@ -39748,7 +39748,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD17" s="172"/>
+      <c r="AD17" s="162"/>
     </row>
     <row r="18" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -39838,7 +39838,7 @@
         <f>SUM(E18:AB18)*D18</f>
         <v>0</v>
       </c>
-      <c r="AD18" s="171">
+      <c r="AD18" s="161">
         <v>0</v>
       </c>
     </row>
@@ -39954,7 +39954,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD19" s="172"/>
+      <c r="AD19" s="162"/>
     </row>
     <row r="20" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -40044,7 +40044,7 @@
         <f>SUM(E20:AB20)*D20</f>
         <v>0</v>
       </c>
-      <c r="AD20" s="171">
+      <c r="AD20" s="161">
         <v>0</v>
       </c>
     </row>
@@ -40160,7 +40160,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD21" s="172"/>
+      <c r="AD21" s="162"/>
     </row>
     <row r="22" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -40269,7 +40269,7 @@
         <f t="shared" ref="AC22" si="10">SUM(E22:AB22)</f>
         <v>54773.4</v>
       </c>
-      <c r="AD22" s="179" t="s">
+      <c r="AD22" s="163" t="s">
         <v>45</v>
       </c>
     </row>
@@ -40380,7 +40380,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD23" s="180"/>
+      <c r="AD23" s="164"/>
     </row>
     <row r="24" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
@@ -40537,32 +40537,32 @@
       <c r="D26" s="68" t="s">
         <v>37</v>
       </c>
-      <c r="E26" s="157" t="s">
+      <c r="E26" s="159" t="s">
         <v>50</v>
       </c>
-      <c r="F26" s="154"/>
-      <c r="G26" s="154"/>
-      <c r="H26" s="154"/>
-      <c r="I26" s="154"/>
-      <c r="J26" s="154"/>
-      <c r="K26" s="154"/>
-      <c r="L26" s="154"/>
-      <c r="M26" s="154"/>
-      <c r="N26" s="154"/>
-      <c r="O26" s="154"/>
-      <c r="P26" s="154"/>
-      <c r="Q26" s="154"/>
-      <c r="R26" s="154"/>
-      <c r="S26" s="154"/>
-      <c r="T26" s="154"/>
-      <c r="U26" s="154"/>
-      <c r="V26" s="154"/>
-      <c r="W26" s="154"/>
-      <c r="X26" s="154"/>
-      <c r="Y26" s="154"/>
-      <c r="Z26" s="154"/>
-      <c r="AA26" s="154"/>
-      <c r="AB26" s="154"/>
+      <c r="F26" s="160"/>
+      <c r="G26" s="160"/>
+      <c r="H26" s="160"/>
+      <c r="I26" s="160"/>
+      <c r="J26" s="160"/>
+      <c r="K26" s="160"/>
+      <c r="L26" s="160"/>
+      <c r="M26" s="160"/>
+      <c r="N26" s="160"/>
+      <c r="O26" s="160"/>
+      <c r="P26" s="160"/>
+      <c r="Q26" s="160"/>
+      <c r="R26" s="160"/>
+      <c r="S26" s="160"/>
+      <c r="T26" s="160"/>
+      <c r="U26" s="160"/>
+      <c r="V26" s="160"/>
+      <c r="W26" s="160"/>
+      <c r="X26" s="160"/>
+      <c r="Y26" s="160"/>
+      <c r="Z26" s="160"/>
+      <c r="AA26" s="160"/>
+      <c r="AB26" s="160"/>
       <c r="AC26" s="61"/>
       <c r="AD26" s="89"/>
     </row>
@@ -40654,7 +40654,7 @@
         <f>SUM(E27:AB27)*D27</f>
         <v>0</v>
       </c>
-      <c r="AD27" s="171">
+      <c r="AD27" s="161">
         <v>0</v>
       </c>
     </row>
@@ -40770,7 +40770,7 @@
         <f t="shared" ref="AC28" si="14">SUM(E28:AB28)</f>
         <v>0</v>
       </c>
-      <c r="AD28" s="172"/>
+      <c r="AD28" s="162"/>
     </row>
     <row r="29" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
@@ -40860,7 +40860,7 @@
         <f>SUM(E29:AB29)*D29</f>
         <v>5600</v>
       </c>
-      <c r="AD29" s="171">
+      <c r="AD29" s="161">
         <f>AC29</f>
         <v>5600</v>
       </c>
@@ -40977,7 +40977,7 @@
         <f t="shared" ref="AC30" si="16">SUM(E30:AB30)</f>
         <v>0</v>
       </c>
-      <c r="AD30" s="172"/>
+      <c r="AD30" s="162"/>
     </row>
     <row r="31" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
@@ -41067,7 +41067,7 @@
         <f>SUM(E31:AB31)*D31</f>
         <v>0</v>
       </c>
-      <c r="AD31" s="171">
+      <c r="AD31" s="161">
         <v>0</v>
       </c>
     </row>
@@ -41183,7 +41183,7 @@
         <f t="shared" ref="AC32" si="18">SUM(E32:AB32)</f>
         <v>0</v>
       </c>
-      <c r="AD32" s="172"/>
+      <c r="AD32" s="162"/>
     </row>
     <row r="33" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -41273,7 +41273,7 @@
         <f>SUM(E33:AB33)*D33</f>
         <v>0</v>
       </c>
-      <c r="AD33" s="181">
+      <c r="AD33" s="165">
         <v>0</v>
       </c>
     </row>
@@ -41389,7 +41389,7 @@
         <f t="shared" ref="AC34" si="20">SUM(E34:AB34)</f>
         <v>0</v>
       </c>
-      <c r="AD34" s="172"/>
+      <c r="AD34" s="162"/>
     </row>
     <row r="35" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -41479,7 +41479,7 @@
         <f>SUM(E35:AB35)*D35</f>
         <v>0</v>
       </c>
-      <c r="AD35" s="171">
+      <c r="AD35" s="161">
         <v>0</v>
       </c>
     </row>
@@ -41595,7 +41595,7 @@
         <f t="shared" ref="AC36" si="22">SUM(E36:AB36)</f>
         <v>0</v>
       </c>
-      <c r="AD36" s="172"/>
+      <c r="AD36" s="162"/>
     </row>
     <row r="37" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -41685,7 +41685,7 @@
         <f>SUM(E37:AB37)*D37</f>
         <v>0</v>
       </c>
-      <c r="AD37" s="171">
+      <c r="AD37" s="161">
         <v>0</v>
       </c>
     </row>
@@ -41801,7 +41801,7 @@
         <f t="shared" ref="AC38" si="24">SUM(E38:AB38)</f>
         <v>0</v>
       </c>
-      <c r="AD38" s="172"/>
+      <c r="AD38" s="162"/>
     </row>
     <row r="39" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
@@ -41891,7 +41891,7 @@
         <f>SUM(E39:AB39)*D39</f>
         <v>0</v>
       </c>
-      <c r="AD39" s="171">
+      <c r="AD39" s="161">
         <v>0</v>
       </c>
     </row>
@@ -42007,7 +42007,7 @@
         <f t="shared" ref="AC40:AC42" si="26">SUM(E40:AB40)</f>
         <v>0</v>
       </c>
-      <c r="AD40" s="172"/>
+      <c r="AD40" s="162"/>
     </row>
     <row r="41" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
@@ -42116,7 +42116,7 @@
         <f t="shared" si="26"/>
         <v>5600</v>
       </c>
-      <c r="AD41" s="162" t="s">
+      <c r="AD41" s="157" t="s">
         <v>45</v>
       </c>
     </row>
@@ -42227,7 +42227,7 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-      <c r="AD42" s="162"/>
+      <c r="AD42" s="157"/>
     </row>
     <row r="43" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
@@ -42380,42 +42380,42 @@
       </c>
       <c r="C45" s="66"/>
       <c r="D45" s="66"/>
-      <c r="E45" s="157" t="s">
+      <c r="E45" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="F45" s="154"/>
-      <c r="G45" s="154"/>
-      <c r="H45" s="154"/>
-      <c r="I45" s="154"/>
-      <c r="J45" s="154"/>
-      <c r="K45" s="154"/>
-      <c r="L45" s="154"/>
-      <c r="M45" s="154"/>
-      <c r="N45" s="154"/>
-      <c r="O45" s="154"/>
-      <c r="P45" s="154"/>
-      <c r="Q45" s="154"/>
-      <c r="R45" s="154"/>
-      <c r="S45" s="154"/>
-      <c r="T45" s="154"/>
-      <c r="U45" s="154"/>
-      <c r="V45" s="154"/>
-      <c r="W45" s="154"/>
-      <c r="X45" s="154"/>
-      <c r="Y45" s="154"/>
-      <c r="Z45" s="154"/>
-      <c r="AA45" s="154"/>
-      <c r="AB45" s="154"/>
+      <c r="F45" s="160"/>
+      <c r="G45" s="160"/>
+      <c r="H45" s="160"/>
+      <c r="I45" s="160"/>
+      <c r="J45" s="160"/>
+      <c r="K45" s="160"/>
+      <c r="L45" s="160"/>
+      <c r="M45" s="160"/>
+      <c r="N45" s="160"/>
+      <c r="O45" s="160"/>
+      <c r="P45" s="160"/>
+      <c r="Q45" s="160"/>
+      <c r="R45" s="160"/>
+      <c r="S45" s="160"/>
+      <c r="T45" s="160"/>
+      <c r="U45" s="160"/>
+      <c r="V45" s="160"/>
+      <c r="W45" s="160"/>
+      <c r="X45" s="160"/>
+      <c r="Y45" s="160"/>
+      <c r="Z45" s="160"/>
+      <c r="AA45" s="160"/>
+      <c r="AB45" s="160"/>
       <c r="AC45" s="61"/>
       <c r="AD45" s="89"/>
     </row>
     <row r="46" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
-      <c r="B46" s="158" t="s">
+      <c r="B46" s="166" t="s">
         <v>40</v>
       </c>
-      <c r="C46" s="159"/>
-      <c r="D46" s="159"/>
+      <c r="C46" s="167"/>
+      <c r="D46" s="167"/>
       <c r="E46" s="12">
         <v>0</v>
       </c>
@@ -42498,11 +42498,11 @@
     </row>
     <row r="47" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
-      <c r="B47" s="160" t="s">
+      <c r="B47" s="153" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="161"/>
-      <c r="D47" s="161"/>
+      <c r="C47" s="154"/>
+      <c r="D47" s="154"/>
       <c r="E47" s="15">
         <v>0</v>
       </c>
@@ -42585,11 +42585,11 @@
     </row>
     <row r="48" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
-      <c r="B48" s="160" t="s">
+      <c r="B48" s="153" t="s">
         <v>47</v>
       </c>
-      <c r="C48" s="161"/>
-      <c r="D48" s="161"/>
+      <c r="C48" s="154"/>
+      <c r="D48" s="154"/>
       <c r="E48" s="15">
         <v>0</v>
       </c>
@@ -42672,11 +42672,11 @@
     </row>
     <row r="49" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
-      <c r="B49" s="160" t="s">
+      <c r="B49" s="153" t="s">
         <v>43</v>
       </c>
-      <c r="C49" s="161"/>
-      <c r="D49" s="161"/>
+      <c r="C49" s="154"/>
+      <c r="D49" s="154"/>
       <c r="E49" s="18">
         <v>0</v>
       </c>
@@ -42903,47 +42903,47 @@
     </row>
     <row r="52" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
-      <c r="B52" s="155" t="s">
+      <c r="B52" s="188" t="s">
         <v>15</v>
       </c>
-      <c r="C52" s="156"/>
-      <c r="D52" s="156"/>
-      <c r="E52" s="157" t="s">
+      <c r="C52" s="189"/>
+      <c r="D52" s="189"/>
+      <c r="E52" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="F52" s="154"/>
-      <c r="G52" s="154"/>
-      <c r="H52" s="154"/>
-      <c r="I52" s="154"/>
-      <c r="J52" s="154"/>
-      <c r="K52" s="154"/>
-      <c r="L52" s="154"/>
-      <c r="M52" s="154"/>
-      <c r="N52" s="154"/>
-      <c r="O52" s="154"/>
-      <c r="P52" s="154"/>
-      <c r="Q52" s="154"/>
-      <c r="R52" s="154"/>
-      <c r="S52" s="154"/>
-      <c r="T52" s="154"/>
-      <c r="U52" s="154"/>
-      <c r="V52" s="154"/>
-      <c r="W52" s="154"/>
-      <c r="X52" s="154"/>
-      <c r="Y52" s="154"/>
-      <c r="Z52" s="154"/>
-      <c r="AA52" s="154"/>
-      <c r="AB52" s="154"/>
+      <c r="F52" s="160"/>
+      <c r="G52" s="160"/>
+      <c r="H52" s="160"/>
+      <c r="I52" s="160"/>
+      <c r="J52" s="160"/>
+      <c r="K52" s="160"/>
+      <c r="L52" s="160"/>
+      <c r="M52" s="160"/>
+      <c r="N52" s="160"/>
+      <c r="O52" s="160"/>
+      <c r="P52" s="160"/>
+      <c r="Q52" s="160"/>
+      <c r="R52" s="160"/>
+      <c r="S52" s="160"/>
+      <c r="T52" s="160"/>
+      <c r="U52" s="160"/>
+      <c r="V52" s="160"/>
+      <c r="W52" s="160"/>
+      <c r="X52" s="160"/>
+      <c r="Y52" s="160"/>
+      <c r="Z52" s="160"/>
+      <c r="AA52" s="160"/>
+      <c r="AB52" s="160"/>
       <c r="AC52" s="61"/>
       <c r="AD52" s="89"/>
     </row>
     <row r="53" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
-      <c r="B53" s="158" t="s">
+      <c r="B53" s="166" t="s">
         <v>16</v>
       </c>
-      <c r="C53" s="159"/>
-      <c r="D53" s="159"/>
+      <c r="C53" s="167"/>
+      <c r="D53" s="167"/>
       <c r="E53" s="12">
         <v>0</v>
       </c>
@@ -43026,11 +43026,11 @@
     </row>
     <row r="54" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="160" t="s">
+      <c r="B54" s="153" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="161"/>
-      <c r="D54" s="161"/>
+      <c r="C54" s="154"/>
+      <c r="D54" s="154"/>
       <c r="E54" s="15">
         <v>0</v>
       </c>
@@ -43113,11 +43113,11 @@
     </row>
     <row r="55" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
-      <c r="B55" s="160" t="s">
+      <c r="B55" s="153" t="s">
         <v>18</v>
       </c>
-      <c r="C55" s="161"/>
-      <c r="D55" s="161"/>
+      <c r="C55" s="154"/>
+      <c r="D55" s="154"/>
       <c r="E55" s="15">
         <v>0</v>
       </c>
@@ -43200,11 +43200,11 @@
     </row>
     <row r="56" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
-      <c r="B56" s="160" t="s">
+      <c r="B56" s="153" t="s">
         <v>18</v>
       </c>
-      <c r="C56" s="161"/>
-      <c r="D56" s="161"/>
+      <c r="C56" s="154"/>
+      <c r="D56" s="154"/>
       <c r="E56" s="18">
         <v>0</v>
       </c>
@@ -43431,47 +43431,47 @@
     </row>
     <row r="59" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
-      <c r="B59" s="166" t="s">
+      <c r="B59" s="171" t="s">
         <v>19</v>
       </c>
-      <c r="C59" s="167"/>
-      <c r="D59" s="167"/>
-      <c r="E59" s="157" t="s">
+      <c r="C59" s="172"/>
+      <c r="D59" s="172"/>
+      <c r="E59" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="F59" s="154"/>
-      <c r="G59" s="154"/>
-      <c r="H59" s="154"/>
-      <c r="I59" s="154"/>
-      <c r="J59" s="154"/>
-      <c r="K59" s="154"/>
-      <c r="L59" s="154"/>
-      <c r="M59" s="154"/>
-      <c r="N59" s="154"/>
-      <c r="O59" s="154"/>
-      <c r="P59" s="154"/>
-      <c r="Q59" s="154"/>
-      <c r="R59" s="154"/>
-      <c r="S59" s="154"/>
-      <c r="T59" s="154"/>
-      <c r="U59" s="154"/>
-      <c r="V59" s="154"/>
-      <c r="W59" s="154"/>
-      <c r="X59" s="154"/>
-      <c r="Y59" s="154"/>
-      <c r="Z59" s="154"/>
-      <c r="AA59" s="154"/>
-      <c r="AB59" s="154"/>
+      <c r="F59" s="160"/>
+      <c r="G59" s="160"/>
+      <c r="H59" s="160"/>
+      <c r="I59" s="160"/>
+      <c r="J59" s="160"/>
+      <c r="K59" s="160"/>
+      <c r="L59" s="160"/>
+      <c r="M59" s="160"/>
+      <c r="N59" s="160"/>
+      <c r="O59" s="160"/>
+      <c r="P59" s="160"/>
+      <c r="Q59" s="160"/>
+      <c r="R59" s="160"/>
+      <c r="S59" s="160"/>
+      <c r="T59" s="160"/>
+      <c r="U59" s="160"/>
+      <c r="V59" s="160"/>
+      <c r="W59" s="160"/>
+      <c r="X59" s="160"/>
+      <c r="Y59" s="160"/>
+      <c r="Z59" s="160"/>
+      <c r="AA59" s="160"/>
+      <c r="AB59" s="160"/>
       <c r="AC59" s="61"/>
       <c r="AD59" s="89"/>
     </row>
     <row r="60" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
-      <c r="B60" s="158" t="s">
+      <c r="B60" s="166" t="s">
         <v>20</v>
       </c>
-      <c r="C60" s="159"/>
-      <c r="D60" s="159"/>
+      <c r="C60" s="167"/>
+      <c r="D60" s="167"/>
       <c r="E60" s="12">
         <v>0</v>
       </c>
@@ -43479,10 +43479,10 @@
         <v>0</v>
       </c>
       <c r="G60" s="13">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H60" s="12">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I60" s="12">
         <v>0</v>
@@ -43546,7 +43546,7 @@
       </c>
       <c r="AC60" s="14">
         <f t="shared" ref="AC60:AC67" si="34">SUM(E60:AB60)</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="AD60" s="122">
         <v>0</v>
@@ -43554,11 +43554,11 @@
     </row>
     <row r="61" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
-      <c r="B61" s="160" t="s">
+      <c r="B61" s="153" t="s">
         <v>41</v>
       </c>
-      <c r="C61" s="161"/>
-      <c r="D61" s="161"/>
+      <c r="C61" s="154"/>
+      <c r="D61" s="154"/>
       <c r="E61" s="15">
         <v>0</v>
       </c>
@@ -43641,11 +43641,11 @@
     </row>
     <row r="62" spans="1:30" ht="15" x14ac:dyDescent="0.3">
       <c r="A62" s="3"/>
-      <c r="B62" s="160" t="s">
+      <c r="B62" s="153" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="161"/>
-      <c r="D62" s="161"/>
+      <c r="C62" s="154"/>
+      <c r="D62" s="154"/>
       <c r="E62" s="15">
         <v>0</v>
       </c>
@@ -43743,11 +43743,11 @@
       </c>
       <c r="G63" s="64">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H63" s="63">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I63" s="63">
         <f t="shared" si="35"/>
@@ -43831,7 +43831,7 @@
       </c>
       <c r="AC63" s="65">
         <f t="shared" si="34"/>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="AD63" s="93">
         <f>SUM(AD60:AD62)</f>
@@ -43887,11 +43887,11 @@
       </c>
       <c r="G65" s="103">
         <f t="shared" si="36"/>
-        <v>5792.6</v>
+        <v>6792.6</v>
       </c>
       <c r="H65" s="103">
         <f t="shared" si="36"/>
-        <v>5792.6</v>
+        <v>6792.6</v>
       </c>
       <c r="I65" s="103">
         <f t="shared" si="36"/>
@@ -43975,9 +43975,9 @@
       </c>
       <c r="AC65" s="104">
         <f>SUM(E65:AB65)</f>
-        <v>60373.4</v>
-      </c>
-      <c r="AD65" s="169"/>
+        <v>62373.4</v>
+      </c>
+      <c r="AD65" s="174"/>
     </row>
     <row r="66" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
@@ -44086,7 +44086,7 @@
         <f t="shared" ref="AC66" si="38">SUM(E66:AB66)</f>
         <v>0</v>
       </c>
-      <c r="AD66" s="162"/>
+      <c r="AD66" s="157"/>
     </row>
     <row r="67" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
@@ -44105,11 +44105,11 @@
       </c>
       <c r="G67" s="107">
         <f t="shared" si="39"/>
-        <v>5792.6</v>
+        <v>6792.6</v>
       </c>
       <c r="H67" s="107">
         <f t="shared" si="39"/>
-        <v>5792.6</v>
+        <v>6792.6</v>
       </c>
       <c r="I67" s="107">
         <f t="shared" si="39"/>
@@ -44193,9 +44193,9 @@
       </c>
       <c r="AC67" s="108">
         <f t="shared" si="34"/>
-        <v>60373.4</v>
-      </c>
-      <c r="AD67" s="162"/>
+        <v>62373.4</v>
+      </c>
+      <c r="AD67" s="157"/>
     </row>
     <row r="68" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
@@ -44214,94 +44214,94 @@
       </c>
       <c r="G68" s="111">
         <f t="shared" ref="G68:AB68" si="40">F68+G67</f>
-        <v>19824.2</v>
+        <v>20824.2</v>
       </c>
       <c r="H68" s="111">
         <f t="shared" si="40"/>
-        <v>25616.800000000003</v>
+        <v>27616.800000000003</v>
       </c>
       <c r="I68" s="111">
         <f t="shared" si="40"/>
-        <v>31409.4</v>
+        <v>33409.4</v>
       </c>
       <c r="J68" s="111">
         <f t="shared" si="40"/>
-        <v>38650.400000000001</v>
+        <v>40650.400000000001</v>
       </c>
       <c r="K68" s="111">
         <f t="shared" si="40"/>
-        <v>45891.4</v>
+        <v>47891.4</v>
       </c>
       <c r="L68" s="111">
         <f t="shared" si="40"/>
-        <v>53132.4</v>
+        <v>55132.4</v>
       </c>
       <c r="M68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="N68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="O68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="P68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="Q68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="R68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="S68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="T68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="U68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="V68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="W68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="X68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="Y68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="Z68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="AA68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="AB68" s="111">
         <f t="shared" si="40"/>
-        <v>60373.4</v>
+        <v>62373.4</v>
       </c>
       <c r="AC68" s="112"/>
-      <c r="AD68" s="163"/>
+      <c r="AD68" s="168"/>
     </row>
     <row r="69" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
@@ -44342,31 +44342,31 @@
       </c>
       <c r="C70" s="60"/>
       <c r="D70" s="60"/>
-      <c r="E70" s="153"/>
-      <c r="F70" s="154"/>
-      <c r="G70" s="154"/>
-      <c r="H70" s="154"/>
-      <c r="I70" s="154"/>
-      <c r="J70" s="154"/>
-      <c r="K70" s="154"/>
-      <c r="L70" s="154"/>
-      <c r="M70" s="154"/>
-      <c r="N70" s="154"/>
-      <c r="O70" s="154"/>
-      <c r="P70" s="154"/>
-      <c r="Q70" s="154"/>
-      <c r="R70" s="154"/>
-      <c r="S70" s="154"/>
-      <c r="T70" s="154"/>
-      <c r="U70" s="154"/>
-      <c r="V70" s="154"/>
-      <c r="W70" s="154"/>
-      <c r="X70" s="154"/>
-      <c r="Y70" s="154"/>
-      <c r="Z70" s="154"/>
-      <c r="AA70" s="154"/>
-      <c r="AB70" s="154"/>
-      <c r="AC70" s="154"/>
+      <c r="E70" s="187"/>
+      <c r="F70" s="160"/>
+      <c r="G70" s="160"/>
+      <c r="H70" s="160"/>
+      <c r="I70" s="160"/>
+      <c r="J70" s="160"/>
+      <c r="K70" s="160"/>
+      <c r="L70" s="160"/>
+      <c r="M70" s="160"/>
+      <c r="N70" s="160"/>
+      <c r="O70" s="160"/>
+      <c r="P70" s="160"/>
+      <c r="Q70" s="160"/>
+      <c r="R70" s="160"/>
+      <c r="S70" s="160"/>
+      <c r="T70" s="160"/>
+      <c r="U70" s="160"/>
+      <c r="V70" s="160"/>
+      <c r="W70" s="160"/>
+      <c r="X70" s="160"/>
+      <c r="Y70" s="160"/>
+      <c r="Z70" s="160"/>
+      <c r="AA70" s="160"/>
+      <c r="AB70" s="160"/>
+      <c r="AC70" s="160"/>
       <c r="AD70" s="89"/>
     </row>
     <row r="71" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
@@ -44378,35 +44378,35 @@
       <c r="D71" s="142">
         <v>0</v>
       </c>
-      <c r="E71" s="175">
+      <c r="E71" s="178">
         <f>D71-E72</f>
         <v>0</v>
       </c>
-      <c r="F71" s="176"/>
-      <c r="G71" s="176"/>
-      <c r="H71" s="176"/>
-      <c r="I71" s="176"/>
-      <c r="J71" s="176"/>
-      <c r="K71" s="176"/>
-      <c r="L71" s="176"/>
-      <c r="M71" s="176"/>
-      <c r="N71" s="176"/>
-      <c r="O71" s="176"/>
-      <c r="P71" s="176"/>
-      <c r="Q71" s="176"/>
-      <c r="R71" s="176"/>
-      <c r="S71" s="176"/>
-      <c r="T71" s="176"/>
-      <c r="U71" s="176"/>
-      <c r="V71" s="176"/>
-      <c r="W71" s="176"/>
-      <c r="X71" s="176"/>
-      <c r="Y71" s="176"/>
-      <c r="Z71" s="176"/>
-      <c r="AA71" s="176"/>
-      <c r="AB71" s="176"/>
-      <c r="AC71" s="176"/>
-      <c r="AD71" s="171">
+      <c r="F71" s="179"/>
+      <c r="G71" s="179"/>
+      <c r="H71" s="179"/>
+      <c r="I71" s="179"/>
+      <c r="J71" s="179"/>
+      <c r="K71" s="179"/>
+      <c r="L71" s="179"/>
+      <c r="M71" s="179"/>
+      <c r="N71" s="179"/>
+      <c r="O71" s="179"/>
+      <c r="P71" s="179"/>
+      <c r="Q71" s="179"/>
+      <c r="R71" s="179"/>
+      <c r="S71" s="179"/>
+      <c r="T71" s="179"/>
+      <c r="U71" s="179"/>
+      <c r="V71" s="179"/>
+      <c r="W71" s="179"/>
+      <c r="X71" s="179"/>
+      <c r="Y71" s="179"/>
+      <c r="Z71" s="179"/>
+      <c r="AA71" s="179"/>
+      <c r="AB71" s="179"/>
+      <c r="AC71" s="179"/>
+      <c r="AD71" s="161">
         <v>0</v>
       </c>
     </row>
@@ -44419,35 +44419,35 @@
       <c r="D72" s="143">
         <v>0</v>
       </c>
-      <c r="E72" s="177">
+      <c r="E72" s="180">
         <f>D71*D72</f>
         <v>0</v>
       </c>
-      <c r="F72" s="178"/>
-      <c r="G72" s="178"/>
-      <c r="H72" s="178"/>
-      <c r="I72" s="178"/>
-      <c r="J72" s="178"/>
-      <c r="K72" s="178"/>
-      <c r="L72" s="178"/>
-      <c r="M72" s="178"/>
-      <c r="N72" s="178"/>
-      <c r="O72" s="178"/>
-      <c r="P72" s="178"/>
-      <c r="Q72" s="178"/>
-      <c r="R72" s="178"/>
-      <c r="S72" s="178"/>
-      <c r="T72" s="178"/>
-      <c r="U72" s="178"/>
-      <c r="V72" s="178"/>
-      <c r="W72" s="178"/>
-      <c r="X72" s="178"/>
-      <c r="Y72" s="178"/>
-      <c r="Z72" s="178"/>
-      <c r="AA72" s="178"/>
-      <c r="AB72" s="178"/>
-      <c r="AC72" s="178"/>
-      <c r="AD72" s="172"/>
+      <c r="F72" s="181"/>
+      <c r="G72" s="181"/>
+      <c r="H72" s="181"/>
+      <c r="I72" s="181"/>
+      <c r="J72" s="181"/>
+      <c r="K72" s="181"/>
+      <c r="L72" s="181"/>
+      <c r="M72" s="181"/>
+      <c r="N72" s="181"/>
+      <c r="O72" s="181"/>
+      <c r="P72" s="181"/>
+      <c r="Q72" s="181"/>
+      <c r="R72" s="181"/>
+      <c r="S72" s="181"/>
+      <c r="T72" s="181"/>
+      <c r="U72" s="181"/>
+      <c r="V72" s="181"/>
+      <c r="W72" s="181"/>
+      <c r="X72" s="181"/>
+      <c r="Y72" s="181"/>
+      <c r="Z72" s="181"/>
+      <c r="AA72" s="181"/>
+      <c r="AB72" s="181"/>
+      <c r="AC72" s="181"/>
+      <c r="AD72" s="162"/>
     </row>
     <row r="73" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
@@ -44461,76 +44461,76 @@
         <f>223.7*9</f>
         <v>2013.3</v>
       </c>
-      <c r="E73" s="170">
+      <c r="E73" s="175">
         <f>D73-E74</f>
         <v>2013.3</v>
       </c>
-      <c r="F73" s="170"/>
-      <c r="G73" s="170"/>
-      <c r="H73" s="170"/>
-      <c r="I73" s="170"/>
-      <c r="J73" s="170"/>
-      <c r="K73" s="170"/>
-      <c r="L73" s="170"/>
-      <c r="M73" s="170"/>
-      <c r="N73" s="170"/>
-      <c r="O73" s="170"/>
-      <c r="P73" s="170"/>
-      <c r="Q73" s="170"/>
-      <c r="R73" s="170"/>
-      <c r="S73" s="170"/>
-      <c r="T73" s="170"/>
-      <c r="U73" s="170"/>
-      <c r="V73" s="170"/>
-      <c r="W73" s="170"/>
-      <c r="X73" s="170"/>
-      <c r="Y73" s="170"/>
-      <c r="Z73" s="170"/>
-      <c r="AA73" s="170"/>
-      <c r="AB73" s="170"/>
-      <c r="AC73" s="170"/>
-      <c r="AD73" s="171">
+      <c r="F73" s="175"/>
+      <c r="G73" s="175"/>
+      <c r="H73" s="175"/>
+      <c r="I73" s="175"/>
+      <c r="J73" s="175"/>
+      <c r="K73" s="175"/>
+      <c r="L73" s="175"/>
+      <c r="M73" s="175"/>
+      <c r="N73" s="175"/>
+      <c r="O73" s="175"/>
+      <c r="P73" s="175"/>
+      <c r="Q73" s="175"/>
+      <c r="R73" s="175"/>
+      <c r="S73" s="175"/>
+      <c r="T73" s="175"/>
+      <c r="U73" s="175"/>
+      <c r="V73" s="175"/>
+      <c r="W73" s="175"/>
+      <c r="X73" s="175"/>
+      <c r="Y73" s="175"/>
+      <c r="Z73" s="175"/>
+      <c r="AA73" s="175"/>
+      <c r="AB73" s="175"/>
+      <c r="AC73" s="175"/>
+      <c r="AD73" s="161">
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
-      <c r="B74" s="173" t="s">
+      <c r="B74" s="176" t="s">
         <v>57</v>
       </c>
-      <c r="C74" s="174"/>
+      <c r="C74" s="177"/>
       <c r="D74" s="121">
         <v>0</v>
       </c>
-      <c r="E74" s="170">
+      <c r="E74" s="175">
         <f>D73*D74</f>
         <v>0</v>
       </c>
-      <c r="F74" s="170"/>
-      <c r="G74" s="170"/>
-      <c r="H74" s="170"/>
-      <c r="I74" s="170"/>
-      <c r="J74" s="170"/>
-      <c r="K74" s="170"/>
-      <c r="L74" s="170"/>
-      <c r="M74" s="170"/>
-      <c r="N74" s="170"/>
-      <c r="O74" s="170"/>
-      <c r="P74" s="170"/>
-      <c r="Q74" s="170"/>
-      <c r="R74" s="170"/>
-      <c r="S74" s="170"/>
-      <c r="T74" s="170"/>
-      <c r="U74" s="170"/>
-      <c r="V74" s="170"/>
-      <c r="W74" s="170"/>
-      <c r="X74" s="170"/>
-      <c r="Y74" s="170"/>
-      <c r="Z74" s="170"/>
-      <c r="AA74" s="170"/>
-      <c r="AB74" s="170"/>
-      <c r="AC74" s="170"/>
-      <c r="AD74" s="172"/>
+      <c r="F74" s="175"/>
+      <c r="G74" s="175"/>
+      <c r="H74" s="175"/>
+      <c r="I74" s="175"/>
+      <c r="J74" s="175"/>
+      <c r="K74" s="175"/>
+      <c r="L74" s="175"/>
+      <c r="M74" s="175"/>
+      <c r="N74" s="175"/>
+      <c r="O74" s="175"/>
+      <c r="P74" s="175"/>
+      <c r="Q74" s="175"/>
+      <c r="R74" s="175"/>
+      <c r="S74" s="175"/>
+      <c r="T74" s="175"/>
+      <c r="U74" s="175"/>
+      <c r="V74" s="175"/>
+      <c r="W74" s="175"/>
+      <c r="X74" s="175"/>
+      <c r="Y74" s="175"/>
+      <c r="Z74" s="175"/>
+      <c r="AA74" s="175"/>
+      <c r="AB74" s="175"/>
+      <c r="AC74" s="175"/>
+      <c r="AD74" s="162"/>
     </row>
     <row r="75" spans="1:30" ht="15" x14ac:dyDescent="0.3">
       <c r="A75" s="3"/>
@@ -44543,35 +44543,35 @@
       <c r="D75" s="117">
         <v>0</v>
       </c>
-      <c r="E75" s="168">
+      <c r="E75" s="173">
         <f>D75</f>
         <v>0</v>
       </c>
-      <c r="F75" s="168"/>
-      <c r="G75" s="168"/>
-      <c r="H75" s="168"/>
-      <c r="I75" s="168"/>
-      <c r="J75" s="168"/>
-      <c r="K75" s="168"/>
-      <c r="L75" s="168"/>
-      <c r="M75" s="168"/>
-      <c r="N75" s="168"/>
-      <c r="O75" s="168"/>
-      <c r="P75" s="168"/>
-      <c r="Q75" s="168"/>
-      <c r="R75" s="168"/>
-      <c r="S75" s="168"/>
-      <c r="T75" s="168"/>
-      <c r="U75" s="168"/>
-      <c r="V75" s="168"/>
-      <c r="W75" s="168"/>
-      <c r="X75" s="168"/>
-      <c r="Y75" s="168"/>
-      <c r="Z75" s="168"/>
-      <c r="AA75" s="168"/>
-      <c r="AB75" s="168"/>
-      <c r="AC75" s="168"/>
-      <c r="AD75" s="162" t="s">
+      <c r="F75" s="173"/>
+      <c r="G75" s="173"/>
+      <c r="H75" s="173"/>
+      <c r="I75" s="173"/>
+      <c r="J75" s="173"/>
+      <c r="K75" s="173"/>
+      <c r="L75" s="173"/>
+      <c r="M75" s="173"/>
+      <c r="N75" s="173"/>
+      <c r="O75" s="173"/>
+      <c r="P75" s="173"/>
+      <c r="Q75" s="173"/>
+      <c r="R75" s="173"/>
+      <c r="S75" s="173"/>
+      <c r="T75" s="173"/>
+      <c r="U75" s="173"/>
+      <c r="V75" s="173"/>
+      <c r="W75" s="173"/>
+      <c r="X75" s="173"/>
+      <c r="Y75" s="173"/>
+      <c r="Z75" s="173"/>
+      <c r="AA75" s="173"/>
+      <c r="AB75" s="173"/>
+      <c r="AC75" s="173"/>
+      <c r="AD75" s="157" t="s">
         <v>54</v>
       </c>
     </row>
@@ -44582,70 +44582,70 @@
       </c>
       <c r="C76" s="119"/>
       <c r="D76" s="119"/>
-      <c r="E76" s="164"/>
-      <c r="F76" s="165"/>
-      <c r="G76" s="165"/>
-      <c r="H76" s="165"/>
-      <c r="I76" s="165"/>
-      <c r="J76" s="165"/>
-      <c r="K76" s="165"/>
-      <c r="L76" s="165"/>
-      <c r="M76" s="165"/>
-      <c r="N76" s="165"/>
-      <c r="O76" s="165"/>
-      <c r="P76" s="165"/>
-      <c r="Q76" s="165"/>
-      <c r="R76" s="165"/>
-      <c r="S76" s="165"/>
-      <c r="T76" s="165"/>
-      <c r="U76" s="165"/>
-      <c r="V76" s="165"/>
-      <c r="W76" s="165"/>
-      <c r="X76" s="165"/>
-      <c r="Y76" s="165"/>
-      <c r="Z76" s="165"/>
-      <c r="AA76" s="165"/>
-      <c r="AB76" s="165"/>
+      <c r="E76" s="169"/>
+      <c r="F76" s="170"/>
+      <c r="G76" s="170"/>
+      <c r="H76" s="170"/>
+      <c r="I76" s="170"/>
+      <c r="J76" s="170"/>
+      <c r="K76" s="170"/>
+      <c r="L76" s="170"/>
+      <c r="M76" s="170"/>
+      <c r="N76" s="170"/>
+      <c r="O76" s="170"/>
+      <c r="P76" s="170"/>
+      <c r="Q76" s="170"/>
+      <c r="R76" s="170"/>
+      <c r="S76" s="170"/>
+      <c r="T76" s="170"/>
+      <c r="U76" s="170"/>
+      <c r="V76" s="170"/>
+      <c r="W76" s="170"/>
+      <c r="X76" s="170"/>
+      <c r="Y76" s="170"/>
+      <c r="Z76" s="170"/>
+      <c r="AA76" s="170"/>
+      <c r="AB76" s="170"/>
       <c r="AC76" s="120">
         <f>D73+D75+D71</f>
         <v>2013.3</v>
       </c>
-      <c r="AD76" s="163"/>
+      <c r="AD76" s="168"/>
     </row>
     <row r="77" spans="1:30" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
-      <c r="B77" s="147" t="s">
+      <c r="B77" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="C77" s="148"/>
+      <c r="C77" s="184"/>
       <c r="D77" s="88"/>
-      <c r="E77" s="149"/>
-      <c r="F77" s="148"/>
-      <c r="G77" s="148"/>
-      <c r="H77" s="148"/>
-      <c r="I77" s="148"/>
-      <c r="J77" s="148"/>
-      <c r="K77" s="148"/>
-      <c r="L77" s="148"/>
-      <c r="M77" s="148"/>
-      <c r="N77" s="148"/>
-      <c r="O77" s="148"/>
-      <c r="P77" s="148"/>
-      <c r="Q77" s="148"/>
-      <c r="R77" s="148"/>
-      <c r="S77" s="148"/>
-      <c r="T77" s="148"/>
-      <c r="U77" s="148"/>
-      <c r="V77" s="148"/>
-      <c r="W77" s="148"/>
-      <c r="X77" s="148"/>
-      <c r="Y77" s="148"/>
-      <c r="Z77" s="148"/>
-      <c r="AA77" s="148"/>
-      <c r="AB77" s="148"/>
+      <c r="E77" s="185"/>
+      <c r="F77" s="184"/>
+      <c r="G77" s="184"/>
+      <c r="H77" s="184"/>
+      <c r="I77" s="184"/>
+      <c r="J77" s="184"/>
+      <c r="K77" s="184"/>
+      <c r="L77" s="184"/>
+      <c r="M77" s="184"/>
+      <c r="N77" s="184"/>
+      <c r="O77" s="184"/>
+      <c r="P77" s="184"/>
+      <c r="Q77" s="184"/>
+      <c r="R77" s="184"/>
+      <c r="S77" s="184"/>
+      <c r="T77" s="184"/>
+      <c r="U77" s="184"/>
+      <c r="V77" s="184"/>
+      <c r="W77" s="184"/>
+      <c r="X77" s="184"/>
+      <c r="Y77" s="184"/>
+      <c r="Z77" s="184"/>
+      <c r="AA77" s="184"/>
+      <c r="AB77" s="184"/>
       <c r="AC77" s="94">
         <f>AC76+AC67</f>
-        <v>62386.700000000004</v>
+        <v>64386.700000000004</v>
       </c>
       <c r="AD77" s="95">
         <f>AD73+AD63+AD57+AD50+AD43+AD24</f>
@@ -44716,10 +44716,10 @@
     </row>
     <row r="80" spans="1:30" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
-      <c r="B80" s="150" t="s">
+      <c r="B80" s="186" t="s">
         <v>27</v>
       </c>
-      <c r="C80" s="151"/>
+      <c r="C80" s="147"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
@@ -44849,10 +44849,10 @@
     </row>
     <row r="84" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A84" s="1"/>
-      <c r="B84" s="152" t="s">
+      <c r="B84" s="146" t="s">
         <v>32</v>
       </c>
-      <c r="C84" s="151"/>
+      <c r="C84" s="147"/>
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
@@ -44881,10 +44881,10 @@
     </row>
     <row r="85" spans="1:29" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1"/>
-      <c r="B85" s="188" t="s">
+      <c r="B85" s="155" t="s">
         <v>33</v>
       </c>
-      <c r="C85" s="151"/>
+      <c r="C85" s="147"/>
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
@@ -44944,10 +44944,10 @@
     </row>
     <row r="87" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
-      <c r="B87" s="189" t="s">
+      <c r="B87" s="156" t="s">
         <v>56</v>
       </c>
-      <c r="C87" s="151"/>
+      <c r="C87" s="147"/>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
@@ -44976,10 +44976,10 @@
     </row>
     <row r="88" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
-      <c r="B88" s="183" t="s">
+      <c r="B88" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="C88" s="151"/>
+      <c r="C88" s="147"/>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
       <c r="G88" s="1"/>
@@ -45008,8 +45008,8 @@
     </row>
     <row r="89" spans="1:29" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
-      <c r="B89" s="151"/>
-      <c r="C89" s="151"/>
+      <c r="B89" s="147"/>
+      <c r="C89" s="147"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
@@ -45069,10 +45069,10 @@
     </row>
     <row r="91" spans="1:29" ht="15" x14ac:dyDescent="0.3">
       <c r="A91" s="1"/>
-      <c r="B91" s="152" t="s">
+      <c r="B91" s="146" t="s">
         <v>59</v>
       </c>
-      <c r="C91" s="151"/>
+      <c r="C91" s="147"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
       <c r="G91" s="1"/>
@@ -45101,10 +45101,10 @@
     </row>
     <row r="92" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A92" s="1"/>
-      <c r="B92" s="183" t="s">
+      <c r="B92" s="148" t="s">
         <v>55</v>
       </c>
-      <c r="C92" s="151"/>
+      <c r="C92" s="147"/>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
@@ -45133,8 +45133,8 @@
     </row>
     <row r="93" spans="1:29" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
-      <c r="B93" s="151"/>
-      <c r="C93" s="151"/>
+      <c r="B93" s="147"/>
+      <c r="C93" s="147"/>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
@@ -45163,10 +45163,10 @@
     </row>
     <row r="94" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
-      <c r="B94" s="152" t="s">
+      <c r="B94" s="146" t="s">
         <v>66</v>
       </c>
-      <c r="C94" s="151"/>
+      <c r="C94" s="147"/>
       <c r="D94" s="4"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
@@ -45196,10 +45196,10 @@
     </row>
     <row r="95" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A95" s="1"/>
-      <c r="B95" s="183" t="s">
+      <c r="B95" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="C95" s="151"/>
+      <c r="C95" s="147"/>
       <c r="D95" s="4"/>
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
@@ -45229,8 +45229,8 @@
     </row>
     <row r="96" spans="1:29" ht="14.25" x14ac:dyDescent="0.3">
       <c r="A96" s="1"/>
-      <c r="B96" s="151"/>
-      <c r="C96" s="151"/>
+      <c r="B96" s="147"/>
+      <c r="C96" s="147"/>
       <c r="D96" s="1"/>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
@@ -74369,43 +74369,17 @@
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B95:C96"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:D3"/>
-    <mergeCell ref="AC3:AC4"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B88:C89"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C93"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="AD3:AD4"/>
-    <mergeCell ref="E4:AB4"/>
-    <mergeCell ref="E26:AB26"/>
-    <mergeCell ref="AD27:AD28"/>
-    <mergeCell ref="E5:AB5"/>
-    <mergeCell ref="AD6:AD7"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="AD10:AD11"/>
-    <mergeCell ref="AD12:AD13"/>
-    <mergeCell ref="AD14:AD15"/>
-    <mergeCell ref="AD39:AD40"/>
-    <mergeCell ref="AD16:AD17"/>
-    <mergeCell ref="AD18:AD19"/>
-    <mergeCell ref="AD20:AD21"/>
-    <mergeCell ref="AD22:AD23"/>
-    <mergeCell ref="AD29:AD30"/>
-    <mergeCell ref="AD31:AD32"/>
-    <mergeCell ref="AD33:AD34"/>
-    <mergeCell ref="AD35:AD36"/>
-    <mergeCell ref="AD37:AD38"/>
-    <mergeCell ref="AD41:AD42"/>
-    <mergeCell ref="E45:AB45"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B1:AC1"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="E77:AB77"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="E70:AC70"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="E52:AB52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B55:D55"/>
     <mergeCell ref="AD75:AD76"/>
     <mergeCell ref="E76:AB76"/>
     <mergeCell ref="B59:D59"/>
@@ -74422,17 +74396,43 @@
     <mergeCell ref="E71:AC71"/>
     <mergeCell ref="E72:AC72"/>
     <mergeCell ref="AD71:AD72"/>
-    <mergeCell ref="B1:AC1"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="E77:AB77"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="E70:AC70"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="E52:AB52"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="AD41:AD42"/>
+    <mergeCell ref="E45:AB45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="AD39:AD40"/>
+    <mergeCell ref="AD16:AD17"/>
+    <mergeCell ref="AD18:AD19"/>
+    <mergeCell ref="AD20:AD21"/>
+    <mergeCell ref="AD22:AD23"/>
+    <mergeCell ref="AD29:AD30"/>
+    <mergeCell ref="AD31:AD32"/>
+    <mergeCell ref="AD33:AD34"/>
+    <mergeCell ref="AD35:AD36"/>
+    <mergeCell ref="AD37:AD38"/>
+    <mergeCell ref="AD3:AD4"/>
+    <mergeCell ref="E4:AB4"/>
+    <mergeCell ref="E26:AB26"/>
+    <mergeCell ref="AD27:AD28"/>
+    <mergeCell ref="E5:AB5"/>
+    <mergeCell ref="AD6:AD7"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="AD10:AD11"/>
+    <mergeCell ref="AD12:AD13"/>
+    <mergeCell ref="AD14:AD15"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B95:C96"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:D3"/>
+    <mergeCell ref="AC3:AC4"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B88:C89"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C93"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B87:C87"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="59" orientation="landscape" r:id="rId1"/>

</xml_diff>